<commit_message>
style: move global export to new global metrics component
</commit_message>
<xml_diff>
--- a/client/src/assets/CPAT_METRICS_TEMPLATE.xlsx
+++ b/client/src/assets/CPAT_METRICS_TEMPLATE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\C-PAT\client\src\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3505453-7350-4253-9453-A96D6F57C7D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D0F1820-D58B-442A-A1DF-81642F9CF750}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5000" yWindow="1880" windowWidth="29190" windowHeight="18060" xr2:uid="{FE1367BE-B521-41BF-8347-968009F83E3B}"/>
+    <workbookView xWindow="5680" yWindow="2560" windowWidth="33570" windowHeight="18060" xr2:uid="{FE1367BE-B521-41BF-8347-968009F83E3B}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
feat: add total open findings counts to global metrics export
</commit_message>
<xml_diff>
--- a/client/src/assets/CPAT_METRICS_TEMPLATE.xlsx
+++ b/client/src/assets/CPAT_METRICS_TEMPLATE.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\C-PAT\client\src\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D0F1820-D58B-442A-A1DF-81642F9CF750}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C5E5DE7-587E-486C-9200-8B5AC937B5D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5680" yWindow="2560" windowWidth="33570" windowHeight="18060" xr2:uid="{FE1367BE-B521-41BF-8347-968009F83E3B}"/>
+    <workbookView xWindow="24560" yWindow="1760" windowWidth="48060" windowHeight="18060" xr2:uid="{FE1367BE-B521-41BF-8347-968009F83E3B}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t xml:space="preserve">Year </t>
   </si>
@@ -121,6 +121,15 @@
   <si>
     <t>POAM Coverage (ACAS) % CAT III 90+ Days</t>
   </si>
+  <si>
+    <t>Open Findings CAT I (Total)</t>
+  </si>
+  <si>
+    <t>Open Findings CAT II (Total)</t>
+  </si>
+  <si>
+    <t>Open Findings CAT III (Total)</t>
+  </si>
 </sst>
 </file>
 
@@ -187,7 +196,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -225,6 +234,15 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -240,7 +258,7 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -583,7 +601,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FC4E6CA-B04F-4BFD-ADE5-E64E7B1F6F62}">
-  <dimension ref="A1:Z100"/>
+  <dimension ref="A1:AC100"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="21.453125" customWidth="1"/>
@@ -601,10 +619,10 @@
     <col min="15" max="16" width="19.54296875" customWidth="1"/>
     <col min="17" max="17" width="16.81640625" customWidth="1"/>
     <col min="18" max="23" width="25.6328125" customWidth="1"/>
-    <col min="24" max="26" width="23.1796875" customWidth="1"/>
+    <col min="24" max="29" width="23.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="18.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:29" ht="18.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
         <v>23</v>
       </c>
@@ -633,8 +651,11 @@
       <c r="X1" s="4"/>
       <c r="Y1" s="4"/>
       <c r="Z1" s="4"/>
-    </row>
-    <row r="2" spans="1:26" ht="67.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA1" s="4"/>
+      <c r="AB1" s="4"/>
+      <c r="AC1" s="4"/>
+    </row>
+    <row r="2" spans="1:29" ht="67.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>12</v>
       </c>
@@ -687,34 +708,43 @@
         <v>19</v>
       </c>
       <c r="R2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="S2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="U2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="S2" s="1" t="s">
+      <c r="V2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="T2" s="1" t="s">
+      <c r="W2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="U2" s="1" t="s">
+      <c r="X2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="V2" s="1" t="s">
+      <c r="Y2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="W2" s="1" t="s">
+      <c r="Z2" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="X2" s="1" t="s">
+      <c r="AA2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="Y2" s="1" t="s">
+      <c r="AB2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="Z2" s="1" t="s">
+      <c r="AC2" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -741,8 +771,11 @@
       <c r="X3" s="2"/>
       <c r="Y3" s="2"/>
       <c r="Z3" s="2"/>
-    </row>
-    <row r="4" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA3" s="2"/>
+      <c r="AB3" s="2"/>
+      <c r="AC3" s="2"/>
+    </row>
+    <row r="4" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="3"/>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -769,8 +802,11 @@
       <c r="X4" s="3"/>
       <c r="Y4" s="3"/>
       <c r="Z4" s="3"/>
-    </row>
-    <row r="5" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA4" s="3"/>
+      <c r="AB4" s="3"/>
+      <c r="AC4" s="3"/>
+    </row>
+    <row r="5" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -797,8 +833,11 @@
       <c r="X5" s="2"/>
       <c r="Y5" s="2"/>
       <c r="Z5" s="2"/>
-    </row>
-    <row r="6" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA5" s="2"/>
+      <c r="AB5" s="2"/>
+      <c r="AC5" s="2"/>
+    </row>
+    <row r="6" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
@@ -825,8 +864,11 @@
       <c r="X6" s="3"/>
       <c r="Y6" s="3"/>
       <c r="Z6" s="3"/>
-    </row>
-    <row r="7" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA6" s="3"/>
+      <c r="AB6" s="3"/>
+      <c r="AC6" s="3"/>
+    </row>
+    <row r="7" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -853,8 +895,11 @@
       <c r="X7" s="2"/>
       <c r="Y7" s="2"/>
       <c r="Z7" s="2"/>
-    </row>
-    <row r="8" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA7" s="2"/>
+      <c r="AB7" s="2"/>
+      <c r="AC7" s="2"/>
+    </row>
+    <row r="8" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="3"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
@@ -881,8 +926,11 @@
       <c r="X8" s="3"/>
       <c r="Y8" s="3"/>
       <c r="Z8" s="3"/>
-    </row>
-    <row r="9" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA8" s="3"/>
+      <c r="AB8" s="3"/>
+      <c r="AC8" s="3"/>
+    </row>
+    <row r="9" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -909,8 +957,11 @@
       <c r="X9" s="2"/>
       <c r="Y9" s="2"/>
       <c r="Z9" s="2"/>
-    </row>
-    <row r="10" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA9" s="2"/>
+      <c r="AB9" s="2"/>
+      <c r="AC9" s="2"/>
+    </row>
+    <row r="10" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="3"/>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
@@ -937,8 +988,11 @@
       <c r="X10" s="3"/>
       <c r="Y10" s="3"/>
       <c r="Z10" s="3"/>
-    </row>
-    <row r="11" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA10" s="3"/>
+      <c r="AB10" s="3"/>
+      <c r="AC10" s="3"/>
+    </row>
+    <row r="11" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -965,8 +1019,11 @@
       <c r="X11" s="2"/>
       <c r="Y11" s="2"/>
       <c r="Z11" s="2"/>
-    </row>
-    <row r="12" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA11" s="2"/>
+      <c r="AB11" s="2"/>
+      <c r="AC11" s="2"/>
+    </row>
+    <row r="12" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="3"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
@@ -993,8 +1050,11 @@
       <c r="X12" s="3"/>
       <c r="Y12" s="3"/>
       <c r="Z12" s="3"/>
-    </row>
-    <row r="13" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA12" s="3"/>
+      <c r="AB12" s="3"/>
+      <c r="AC12" s="3"/>
+    </row>
+    <row r="13" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -1021,8 +1081,11 @@
       <c r="X13" s="2"/>
       <c r="Y13" s="2"/>
       <c r="Z13" s="2"/>
-    </row>
-    <row r="14" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA13" s="2"/>
+      <c r="AB13" s="2"/>
+      <c r="AC13" s="2"/>
+    </row>
+    <row r="14" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="3"/>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
@@ -1049,8 +1112,11 @@
       <c r="X14" s="3"/>
       <c r="Y14" s="3"/>
       <c r="Z14" s="3"/>
-    </row>
-    <row r="15" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA14" s="3"/>
+      <c r="AB14" s="3"/>
+      <c r="AC14" s="3"/>
+    </row>
+    <row r="15" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -1077,8 +1143,11 @@
       <c r="X15" s="2"/>
       <c r="Y15" s="2"/>
       <c r="Z15" s="2"/>
-    </row>
-    <row r="16" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA15" s="2"/>
+      <c r="AB15" s="2"/>
+      <c r="AC15" s="2"/>
+    </row>
+    <row r="16" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="3"/>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
@@ -1105,8 +1174,11 @@
       <c r="X16" s="3"/>
       <c r="Y16" s="3"/>
       <c r="Z16" s="3"/>
-    </row>
-    <row r="17" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA16" s="3"/>
+      <c r="AB16" s="3"/>
+      <c r="AC16" s="3"/>
+    </row>
+    <row r="17" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -1133,8 +1205,11 @@
       <c r="X17" s="2"/>
       <c r="Y17" s="2"/>
       <c r="Z17" s="2"/>
-    </row>
-    <row r="18" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA17" s="2"/>
+      <c r="AB17" s="2"/>
+      <c r="AC17" s="2"/>
+    </row>
+    <row r="18" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="3"/>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
@@ -1161,8 +1236,11 @@
       <c r="X18" s="3"/>
       <c r="Y18" s="3"/>
       <c r="Z18" s="3"/>
-    </row>
-    <row r="19" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA18" s="3"/>
+      <c r="AB18" s="3"/>
+      <c r="AC18" s="3"/>
+    </row>
+    <row r="19" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -1189,8 +1267,11 @@
       <c r="X19" s="2"/>
       <c r="Y19" s="2"/>
       <c r="Z19" s="2"/>
-    </row>
-    <row r="20" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA19" s="2"/>
+      <c r="AB19" s="2"/>
+      <c r="AC19" s="2"/>
+    </row>
+    <row r="20" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="3"/>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
@@ -1217,8 +1298,11 @@
       <c r="X20" s="3"/>
       <c r="Y20" s="3"/>
       <c r="Z20" s="3"/>
-    </row>
-    <row r="21" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA20" s="3"/>
+      <c r="AB20" s="3"/>
+      <c r="AC20" s="3"/>
+    </row>
+    <row r="21" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -1245,8 +1329,11 @@
       <c r="X21" s="2"/>
       <c r="Y21" s="2"/>
       <c r="Z21" s="2"/>
-    </row>
-    <row r="22" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA21" s="2"/>
+      <c r="AB21" s="2"/>
+      <c r="AC21" s="2"/>
+    </row>
+    <row r="22" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="3"/>
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
@@ -1273,8 +1360,11 @@
       <c r="X22" s="3"/>
       <c r="Y22" s="3"/>
       <c r="Z22" s="3"/>
-    </row>
-    <row r="23" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA22" s="3"/>
+      <c r="AB22" s="3"/>
+      <c r="AC22" s="3"/>
+    </row>
+    <row r="23" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
@@ -1301,8 +1391,11 @@
       <c r="X23" s="2"/>
       <c r="Y23" s="2"/>
       <c r="Z23" s="2"/>
-    </row>
-    <row r="24" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA23" s="2"/>
+      <c r="AB23" s="2"/>
+      <c r="AC23" s="2"/>
+    </row>
+    <row r="24" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="3"/>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
@@ -1329,8 +1422,11 @@
       <c r="X24" s="3"/>
       <c r="Y24" s="3"/>
       <c r="Z24" s="3"/>
-    </row>
-    <row r="25" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA24" s="3"/>
+      <c r="AB24" s="3"/>
+      <c r="AC24" s="3"/>
+    </row>
+    <row r="25" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
@@ -1357,8 +1453,11 @@
       <c r="X25" s="2"/>
       <c r="Y25" s="2"/>
       <c r="Z25" s="2"/>
-    </row>
-    <row r="26" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA25" s="2"/>
+      <c r="AB25" s="2"/>
+      <c r="AC25" s="2"/>
+    </row>
+    <row r="26" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="3"/>
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
@@ -1385,8 +1484,11 @@
       <c r="X26" s="3"/>
       <c r="Y26" s="3"/>
       <c r="Z26" s="3"/>
-    </row>
-    <row r="27" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA26" s="3"/>
+      <c r="AB26" s="3"/>
+      <c r="AC26" s="3"/>
+    </row>
+    <row r="27" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
@@ -1413,8 +1515,11 @@
       <c r="X27" s="2"/>
       <c r="Y27" s="2"/>
       <c r="Z27" s="2"/>
-    </row>
-    <row r="28" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA27" s="2"/>
+      <c r="AB27" s="2"/>
+      <c r="AC27" s="2"/>
+    </row>
+    <row r="28" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="3"/>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
@@ -1441,8 +1546,11 @@
       <c r="X28" s="3"/>
       <c r="Y28" s="3"/>
       <c r="Z28" s="3"/>
-    </row>
-    <row r="29" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA28" s="3"/>
+      <c r="AB28" s="3"/>
+      <c r="AC28" s="3"/>
+    </row>
+    <row r="29" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
@@ -1469,8 +1577,11 @@
       <c r="X29" s="2"/>
       <c r="Y29" s="2"/>
       <c r="Z29" s="2"/>
-    </row>
-    <row r="30" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA29" s="2"/>
+      <c r="AB29" s="2"/>
+      <c r="AC29" s="2"/>
+    </row>
+    <row r="30" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="3"/>
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
@@ -1497,8 +1608,11 @@
       <c r="X30" s="3"/>
       <c r="Y30" s="3"/>
       <c r="Z30" s="3"/>
-    </row>
-    <row r="31" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA30" s="3"/>
+      <c r="AB30" s="3"/>
+      <c r="AC30" s="3"/>
+    </row>
+    <row r="31" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
@@ -1525,8 +1639,11 @@
       <c r="X31" s="2"/>
       <c r="Y31" s="2"/>
       <c r="Z31" s="2"/>
-    </row>
-    <row r="32" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA31" s="2"/>
+      <c r="AB31" s="2"/>
+      <c r="AC31" s="2"/>
+    </row>
+    <row r="32" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="3"/>
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
@@ -1553,8 +1670,11 @@
       <c r="X32" s="3"/>
       <c r="Y32" s="3"/>
       <c r="Z32" s="3"/>
-    </row>
-    <row r="33" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA32" s="3"/>
+      <c r="AB32" s="3"/>
+      <c r="AC32" s="3"/>
+    </row>
+    <row r="33" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
@@ -1581,8 +1701,11 @@
       <c r="X33" s="2"/>
       <c r="Y33" s="2"/>
       <c r="Z33" s="2"/>
-    </row>
-    <row r="34" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA33" s="2"/>
+      <c r="AB33" s="2"/>
+      <c r="AC33" s="2"/>
+    </row>
+    <row r="34" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="3"/>
       <c r="B34" s="3"/>
       <c r="C34" s="3"/>
@@ -1609,8 +1732,11 @@
       <c r="X34" s="3"/>
       <c r="Y34" s="3"/>
       <c r="Z34" s="3"/>
-    </row>
-    <row r="35" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA34" s="3"/>
+      <c r="AB34" s="3"/>
+      <c r="AC34" s="3"/>
+    </row>
+    <row r="35" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="2"/>
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
@@ -1637,8 +1763,11 @@
       <c r="X35" s="2"/>
       <c r="Y35" s="2"/>
       <c r="Z35" s="2"/>
-    </row>
-    <row r="36" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA35" s="2"/>
+      <c r="AB35" s="2"/>
+      <c r="AC35" s="2"/>
+    </row>
+    <row r="36" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="3"/>
       <c r="B36" s="3"/>
       <c r="C36" s="3"/>
@@ -1665,8 +1794,11 @@
       <c r="X36" s="3"/>
       <c r="Y36" s="3"/>
       <c r="Z36" s="3"/>
-    </row>
-    <row r="37" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA36" s="3"/>
+      <c r="AB36" s="3"/>
+      <c r="AC36" s="3"/>
+    </row>
+    <row r="37" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
@@ -1693,8 +1825,11 @@
       <c r="X37" s="2"/>
       <c r="Y37" s="2"/>
       <c r="Z37" s="2"/>
-    </row>
-    <row r="38" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA37" s="2"/>
+      <c r="AB37" s="2"/>
+      <c r="AC37" s="2"/>
+    </row>
+    <row r="38" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="3"/>
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
@@ -1721,8 +1856,11 @@
       <c r="X38" s="3"/>
       <c r="Y38" s="3"/>
       <c r="Z38" s="3"/>
-    </row>
-    <row r="39" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA38" s="3"/>
+      <c r="AB38" s="3"/>
+      <c r="AC38" s="3"/>
+    </row>
+    <row r="39" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="2"/>
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
@@ -1749,8 +1887,11 @@
       <c r="X39" s="2"/>
       <c r="Y39" s="2"/>
       <c r="Z39" s="2"/>
-    </row>
-    <row r="40" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA39" s="2"/>
+      <c r="AB39" s="2"/>
+      <c r="AC39" s="2"/>
+    </row>
+    <row r="40" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="3"/>
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
@@ -1777,8 +1918,11 @@
       <c r="X40" s="3"/>
       <c r="Y40" s="3"/>
       <c r="Z40" s="3"/>
-    </row>
-    <row r="41" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA40" s="3"/>
+      <c r="AB40" s="3"/>
+      <c r="AC40" s="3"/>
+    </row>
+    <row r="41" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A41" s="2"/>
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
@@ -1805,8 +1949,11 @@
       <c r="X41" s="2"/>
       <c r="Y41" s="2"/>
       <c r="Z41" s="2"/>
-    </row>
-    <row r="42" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA41" s="2"/>
+      <c r="AB41" s="2"/>
+      <c r="AC41" s="2"/>
+    </row>
+    <row r="42" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="3"/>
       <c r="B42" s="3"/>
       <c r="C42" s="3"/>
@@ -1833,8 +1980,11 @@
       <c r="X42" s="3"/>
       <c r="Y42" s="3"/>
       <c r="Z42" s="3"/>
-    </row>
-    <row r="43" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA42" s="3"/>
+      <c r="AB42" s="3"/>
+      <c r="AC42" s="3"/>
+    </row>
+    <row r="43" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="2"/>
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
@@ -1861,8 +2011,11 @@
       <c r="X43" s="2"/>
       <c r="Y43" s="2"/>
       <c r="Z43" s="2"/>
-    </row>
-    <row r="44" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA43" s="2"/>
+      <c r="AB43" s="2"/>
+      <c r="AC43" s="2"/>
+    </row>
+    <row r="44" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="3"/>
       <c r="B44" s="3"/>
       <c r="C44" s="3"/>
@@ -1889,8 +2042,11 @@
       <c r="X44" s="3"/>
       <c r="Y44" s="3"/>
       <c r="Z44" s="3"/>
-    </row>
-    <row r="45" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA44" s="3"/>
+      <c r="AB44" s="3"/>
+      <c r="AC44" s="3"/>
+    </row>
+    <row r="45" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="2"/>
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
@@ -1917,8 +2073,11 @@
       <c r="X45" s="2"/>
       <c r="Y45" s="2"/>
       <c r="Z45" s="2"/>
-    </row>
-    <row r="46" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA45" s="2"/>
+      <c r="AB45" s="2"/>
+      <c r="AC45" s="2"/>
+    </row>
+    <row r="46" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="3"/>
       <c r="B46" s="3"/>
       <c r="C46" s="3"/>
@@ -1945,8 +2104,11 @@
       <c r="X46" s="3"/>
       <c r="Y46" s="3"/>
       <c r="Z46" s="3"/>
-    </row>
-    <row r="47" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA46" s="3"/>
+      <c r="AB46" s="3"/>
+      <c r="AC46" s="3"/>
+    </row>
+    <row r="47" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="2"/>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
@@ -1973,8 +2135,11 @@
       <c r="X47" s="2"/>
       <c r="Y47" s="2"/>
       <c r="Z47" s="2"/>
-    </row>
-    <row r="48" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA47" s="2"/>
+      <c r="AB47" s="2"/>
+      <c r="AC47" s="2"/>
+    </row>
+    <row r="48" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" s="3"/>
       <c r="B48" s="3"/>
       <c r="C48" s="3"/>
@@ -2001,8 +2166,11 @@
       <c r="X48" s="3"/>
       <c r="Y48" s="3"/>
       <c r="Z48" s="3"/>
-    </row>
-    <row r="49" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA48" s="3"/>
+      <c r="AB48" s="3"/>
+      <c r="AC48" s="3"/>
+    </row>
+    <row r="49" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="2"/>
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
@@ -2029,8 +2197,11 @@
       <c r="X49" s="2"/>
       <c r="Y49" s="2"/>
       <c r="Z49" s="2"/>
-    </row>
-    <row r="50" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA49" s="2"/>
+      <c r="AB49" s="2"/>
+      <c r="AC49" s="2"/>
+    </row>
+    <row r="50" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" s="3"/>
       <c r="B50" s="3"/>
       <c r="C50" s="3"/>
@@ -2057,8 +2228,11 @@
       <c r="X50" s="3"/>
       <c r="Y50" s="3"/>
       <c r="Z50" s="3"/>
-    </row>
-    <row r="51" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA50" s="3"/>
+      <c r="AB50" s="3"/>
+      <c r="AC50" s="3"/>
+    </row>
+    <row r="51" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" s="2"/>
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
@@ -2085,8 +2259,11 @@
       <c r="X51" s="2"/>
       <c r="Y51" s="2"/>
       <c r="Z51" s="2"/>
-    </row>
-    <row r="52" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA51" s="2"/>
+      <c r="AB51" s="2"/>
+      <c r="AC51" s="2"/>
+    </row>
+    <row r="52" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A52" s="3"/>
       <c r="B52" s="3"/>
       <c r="C52" s="3"/>
@@ -2113,8 +2290,11 @@
       <c r="X52" s="3"/>
       <c r="Y52" s="3"/>
       <c r="Z52" s="3"/>
-    </row>
-    <row r="53" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA52" s="3"/>
+      <c r="AB52" s="3"/>
+      <c r="AC52" s="3"/>
+    </row>
+    <row r="53" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A53" s="2"/>
       <c r="B53" s="2"/>
       <c r="C53" s="2"/>
@@ -2141,8 +2321,11 @@
       <c r="X53" s="2"/>
       <c r="Y53" s="2"/>
       <c r="Z53" s="2"/>
-    </row>
-    <row r="54" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA53" s="2"/>
+      <c r="AB53" s="2"/>
+      <c r="AC53" s="2"/>
+    </row>
+    <row r="54" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A54" s="3"/>
       <c r="B54" s="3"/>
       <c r="C54" s="3"/>
@@ -2169,8 +2352,11 @@
       <c r="X54" s="3"/>
       <c r="Y54" s="3"/>
       <c r="Z54" s="3"/>
-    </row>
-    <row r="55" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA54" s="3"/>
+      <c r="AB54" s="3"/>
+      <c r="AC54" s="3"/>
+    </row>
+    <row r="55" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A55" s="2"/>
       <c r="B55" s="2"/>
       <c r="C55" s="2"/>
@@ -2197,8 +2383,11 @@
       <c r="X55" s="2"/>
       <c r="Y55" s="2"/>
       <c r="Z55" s="2"/>
-    </row>
-    <row r="56" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA55" s="2"/>
+      <c r="AB55" s="2"/>
+      <c r="AC55" s="2"/>
+    </row>
+    <row r="56" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A56" s="3"/>
       <c r="B56" s="3"/>
       <c r="C56" s="3"/>
@@ -2225,8 +2414,11 @@
       <c r="X56" s="3"/>
       <c r="Y56" s="3"/>
       <c r="Z56" s="3"/>
-    </row>
-    <row r="57" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA56" s="3"/>
+      <c r="AB56" s="3"/>
+      <c r="AC56" s="3"/>
+    </row>
+    <row r="57" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A57" s="2"/>
       <c r="B57" s="2"/>
       <c r="C57" s="2"/>
@@ -2253,8 +2445,11 @@
       <c r="X57" s="2"/>
       <c r="Y57" s="2"/>
       <c r="Z57" s="2"/>
-    </row>
-    <row r="58" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA57" s="2"/>
+      <c r="AB57" s="2"/>
+      <c r="AC57" s="2"/>
+    </row>
+    <row r="58" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A58" s="3"/>
       <c r="B58" s="3"/>
       <c r="C58" s="3"/>
@@ -2281,8 +2476,11 @@
       <c r="X58" s="3"/>
       <c r="Y58" s="3"/>
       <c r="Z58" s="3"/>
-    </row>
-    <row r="59" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA58" s="3"/>
+      <c r="AB58" s="3"/>
+      <c r="AC58" s="3"/>
+    </row>
+    <row r="59" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A59" s="2"/>
       <c r="B59" s="2"/>
       <c r="C59" s="2"/>
@@ -2309,8 +2507,11 @@
       <c r="X59" s="2"/>
       <c r="Y59" s="2"/>
       <c r="Z59" s="2"/>
-    </row>
-    <row r="60" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA59" s="2"/>
+      <c r="AB59" s="2"/>
+      <c r="AC59" s="2"/>
+    </row>
+    <row r="60" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A60" s="3"/>
       <c r="B60" s="3"/>
       <c r="C60" s="3"/>
@@ -2337,8 +2538,11 @@
       <c r="X60" s="3"/>
       <c r="Y60" s="3"/>
       <c r="Z60" s="3"/>
-    </row>
-    <row r="61" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA60" s="3"/>
+      <c r="AB60" s="3"/>
+      <c r="AC60" s="3"/>
+    </row>
+    <row r="61" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A61" s="2"/>
       <c r="B61" s="2"/>
       <c r="C61" s="2"/>
@@ -2365,8 +2569,11 @@
       <c r="X61" s="2"/>
       <c r="Y61" s="2"/>
       <c r="Z61" s="2"/>
-    </row>
-    <row r="62" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA61" s="2"/>
+      <c r="AB61" s="2"/>
+      <c r="AC61" s="2"/>
+    </row>
+    <row r="62" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A62" s="3"/>
       <c r="B62" s="3"/>
       <c r="C62" s="3"/>
@@ -2393,8 +2600,11 @@
       <c r="X62" s="3"/>
       <c r="Y62" s="3"/>
       <c r="Z62" s="3"/>
-    </row>
-    <row r="63" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA62" s="3"/>
+      <c r="AB62" s="3"/>
+      <c r="AC62" s="3"/>
+    </row>
+    <row r="63" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A63" s="2"/>
       <c r="B63" s="2"/>
       <c r="C63" s="2"/>
@@ -2421,8 +2631,11 @@
       <c r="X63" s="2"/>
       <c r="Y63" s="2"/>
       <c r="Z63" s="2"/>
-    </row>
-    <row r="64" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA63" s="2"/>
+      <c r="AB63" s="2"/>
+      <c r="AC63" s="2"/>
+    </row>
+    <row r="64" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A64" s="3"/>
       <c r="B64" s="3"/>
       <c r="C64" s="3"/>
@@ -2449,8 +2662,11 @@
       <c r="X64" s="3"/>
       <c r="Y64" s="3"/>
       <c r="Z64" s="3"/>
-    </row>
-    <row r="65" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA64" s="3"/>
+      <c r="AB64" s="3"/>
+      <c r="AC64" s="3"/>
+    </row>
+    <row r="65" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A65" s="2"/>
       <c r="B65" s="2"/>
       <c r="C65" s="2"/>
@@ -2477,8 +2693,11 @@
       <c r="X65" s="2"/>
       <c r="Y65" s="2"/>
       <c r="Z65" s="2"/>
-    </row>
-    <row r="66" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA65" s="2"/>
+      <c r="AB65" s="2"/>
+      <c r="AC65" s="2"/>
+    </row>
+    <row r="66" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A66" s="3"/>
       <c r="B66" s="3"/>
       <c r="C66" s="3"/>
@@ -2505,8 +2724,11 @@
       <c r="X66" s="3"/>
       <c r="Y66" s="3"/>
       <c r="Z66" s="3"/>
-    </row>
-    <row r="67" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA66" s="3"/>
+      <c r="AB66" s="3"/>
+      <c r="AC66" s="3"/>
+    </row>
+    <row r="67" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A67" s="2"/>
       <c r="B67" s="2"/>
       <c r="C67" s="2"/>
@@ -2533,8 +2755,11 @@
       <c r="X67" s="2"/>
       <c r="Y67" s="2"/>
       <c r="Z67" s="2"/>
-    </row>
-    <row r="68" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA67" s="2"/>
+      <c r="AB67" s="2"/>
+      <c r="AC67" s="2"/>
+    </row>
+    <row r="68" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A68" s="3"/>
       <c r="B68" s="3"/>
       <c r="C68" s="3"/>
@@ -2561,8 +2786,11 @@
       <c r="X68" s="3"/>
       <c r="Y68" s="3"/>
       <c r="Z68" s="3"/>
-    </row>
-    <row r="69" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA68" s="3"/>
+      <c r="AB68" s="3"/>
+      <c r="AC68" s="3"/>
+    </row>
+    <row r="69" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A69" s="2"/>
       <c r="B69" s="2"/>
       <c r="C69" s="2"/>
@@ -2589,8 +2817,11 @@
       <c r="X69" s="2"/>
       <c r="Y69" s="2"/>
       <c r="Z69" s="2"/>
-    </row>
-    <row r="70" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA69" s="2"/>
+      <c r="AB69" s="2"/>
+      <c r="AC69" s="2"/>
+    </row>
+    <row r="70" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A70" s="3"/>
       <c r="B70" s="3"/>
       <c r="C70" s="3"/>
@@ -2617,8 +2848,11 @@
       <c r="X70" s="3"/>
       <c r="Y70" s="3"/>
       <c r="Z70" s="3"/>
-    </row>
-    <row r="71" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA70" s="3"/>
+      <c r="AB70" s="3"/>
+      <c r="AC70" s="3"/>
+    </row>
+    <row r="71" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A71" s="2"/>
       <c r="B71" s="2"/>
       <c r="C71" s="2"/>
@@ -2645,8 +2879,11 @@
       <c r="X71" s="2"/>
       <c r="Y71" s="2"/>
       <c r="Z71" s="2"/>
-    </row>
-    <row r="72" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA71" s="2"/>
+      <c r="AB71" s="2"/>
+      <c r="AC71" s="2"/>
+    </row>
+    <row r="72" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A72" s="3"/>
       <c r="B72" s="3"/>
       <c r="C72" s="3"/>
@@ -2673,8 +2910,11 @@
       <c r="X72" s="3"/>
       <c r="Y72" s="3"/>
       <c r="Z72" s="3"/>
-    </row>
-    <row r="73" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA72" s="3"/>
+      <c r="AB72" s="3"/>
+      <c r="AC72" s="3"/>
+    </row>
+    <row r="73" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A73" s="2"/>
       <c r="B73" s="2"/>
       <c r="C73" s="2"/>
@@ -2701,8 +2941,11 @@
       <c r="X73" s="2"/>
       <c r="Y73" s="2"/>
       <c r="Z73" s="2"/>
-    </row>
-    <row r="74" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA73" s="2"/>
+      <c r="AB73" s="2"/>
+      <c r="AC73" s="2"/>
+    </row>
+    <row r="74" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A74" s="3"/>
       <c r="B74" s="3"/>
       <c r="C74" s="3"/>
@@ -2729,8 +2972,11 @@
       <c r="X74" s="3"/>
       <c r="Y74" s="3"/>
       <c r="Z74" s="3"/>
-    </row>
-    <row r="75" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA74" s="3"/>
+      <c r="AB74" s="3"/>
+      <c r="AC74" s="3"/>
+    </row>
+    <row r="75" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A75" s="2"/>
       <c r="B75" s="2"/>
       <c r="C75" s="2"/>
@@ -2757,8 +3003,11 @@
       <c r="X75" s="2"/>
       <c r="Y75" s="2"/>
       <c r="Z75" s="2"/>
-    </row>
-    <row r="76" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA75" s="2"/>
+      <c r="AB75" s="2"/>
+      <c r="AC75" s="2"/>
+    </row>
+    <row r="76" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A76" s="3"/>
       <c r="B76" s="3"/>
       <c r="C76" s="3"/>
@@ -2785,8 +3034,11 @@
       <c r="X76" s="3"/>
       <c r="Y76" s="3"/>
       <c r="Z76" s="3"/>
-    </row>
-    <row r="77" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA76" s="3"/>
+      <c r="AB76" s="3"/>
+      <c r="AC76" s="3"/>
+    </row>
+    <row r="77" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A77" s="2"/>
       <c r="B77" s="2"/>
       <c r="C77" s="2"/>
@@ -2813,8 +3065,11 @@
       <c r="X77" s="2"/>
       <c r="Y77" s="2"/>
       <c r="Z77" s="2"/>
-    </row>
-    <row r="78" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA77" s="2"/>
+      <c r="AB77" s="2"/>
+      <c r="AC77" s="2"/>
+    </row>
+    <row r="78" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A78" s="3"/>
       <c r="B78" s="3"/>
       <c r="C78" s="3"/>
@@ -2841,8 +3096,11 @@
       <c r="X78" s="3"/>
       <c r="Y78" s="3"/>
       <c r="Z78" s="3"/>
-    </row>
-    <row r="79" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA78" s="3"/>
+      <c r="AB78" s="3"/>
+      <c r="AC78" s="3"/>
+    </row>
+    <row r="79" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A79" s="2"/>
       <c r="B79" s="2"/>
       <c r="C79" s="2"/>
@@ -2869,8 +3127,11 @@
       <c r="X79" s="2"/>
       <c r="Y79" s="2"/>
       <c r="Z79" s="2"/>
-    </row>
-    <row r="80" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA79" s="2"/>
+      <c r="AB79" s="2"/>
+      <c r="AC79" s="2"/>
+    </row>
+    <row r="80" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A80" s="3"/>
       <c r="B80" s="3"/>
       <c r="C80" s="3"/>
@@ -2897,8 +3158,11 @@
       <c r="X80" s="3"/>
       <c r="Y80" s="3"/>
       <c r="Z80" s="3"/>
-    </row>
-    <row r="81" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA80" s="3"/>
+      <c r="AB80" s="3"/>
+      <c r="AC80" s="3"/>
+    </row>
+    <row r="81" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A81" s="2"/>
       <c r="B81" s="2"/>
       <c r="C81" s="2"/>
@@ -2925,8 +3189,11 @@
       <c r="X81" s="2"/>
       <c r="Y81" s="2"/>
       <c r="Z81" s="2"/>
-    </row>
-    <row r="82" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA81" s="2"/>
+      <c r="AB81" s="2"/>
+      <c r="AC81" s="2"/>
+    </row>
+    <row r="82" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A82" s="3"/>
       <c r="B82" s="3"/>
       <c r="C82" s="3"/>
@@ -2953,8 +3220,11 @@
       <c r="X82" s="3"/>
       <c r="Y82" s="3"/>
       <c r="Z82" s="3"/>
-    </row>
-    <row r="83" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA82" s="3"/>
+      <c r="AB82" s="3"/>
+      <c r="AC82" s="3"/>
+    </row>
+    <row r="83" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A83" s="2"/>
       <c r="B83" s="2"/>
       <c r="C83" s="2"/>
@@ -2981,8 +3251,11 @@
       <c r="X83" s="2"/>
       <c r="Y83" s="2"/>
       <c r="Z83" s="2"/>
-    </row>
-    <row r="84" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA83" s="2"/>
+      <c r="AB83" s="2"/>
+      <c r="AC83" s="2"/>
+    </row>
+    <row r="84" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A84" s="3"/>
       <c r="B84" s="3"/>
       <c r="C84" s="3"/>
@@ -3009,8 +3282,11 @@
       <c r="X84" s="3"/>
       <c r="Y84" s="3"/>
       <c r="Z84" s="3"/>
-    </row>
-    <row r="85" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA84" s="3"/>
+      <c r="AB84" s="3"/>
+      <c r="AC84" s="3"/>
+    </row>
+    <row r="85" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A85" s="2"/>
       <c r="B85" s="2"/>
       <c r="C85" s="2"/>
@@ -3037,8 +3313,11 @@
       <c r="X85" s="2"/>
       <c r="Y85" s="2"/>
       <c r="Z85" s="2"/>
-    </row>
-    <row r="86" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA85" s="2"/>
+      <c r="AB85" s="2"/>
+      <c r="AC85" s="2"/>
+    </row>
+    <row r="86" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A86" s="3"/>
       <c r="B86" s="3"/>
       <c r="C86" s="3"/>
@@ -3065,8 +3344,11 @@
       <c r="X86" s="3"/>
       <c r="Y86" s="3"/>
       <c r="Z86" s="3"/>
-    </row>
-    <row r="87" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA86" s="3"/>
+      <c r="AB86" s="3"/>
+      <c r="AC86" s="3"/>
+    </row>
+    <row r="87" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A87" s="2"/>
       <c r="B87" s="2"/>
       <c r="C87" s="2"/>
@@ -3093,8 +3375,11 @@
       <c r="X87" s="2"/>
       <c r="Y87" s="2"/>
       <c r="Z87" s="2"/>
-    </row>
-    <row r="88" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA87" s="2"/>
+      <c r="AB87" s="2"/>
+      <c r="AC87" s="2"/>
+    </row>
+    <row r="88" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A88" s="3"/>
       <c r="B88" s="3"/>
       <c r="C88" s="3"/>
@@ -3121,8 +3406,11 @@
       <c r="X88" s="3"/>
       <c r="Y88" s="3"/>
       <c r="Z88" s="3"/>
-    </row>
-    <row r="89" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA88" s="3"/>
+      <c r="AB88" s="3"/>
+      <c r="AC88" s="3"/>
+    </row>
+    <row r="89" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A89" s="2"/>
       <c r="B89" s="2"/>
       <c r="C89" s="2"/>
@@ -3149,8 +3437,11 @@
       <c r="X89" s="2"/>
       <c r="Y89" s="2"/>
       <c r="Z89" s="2"/>
-    </row>
-    <row r="90" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA89" s="2"/>
+      <c r="AB89" s="2"/>
+      <c r="AC89" s="2"/>
+    </row>
+    <row r="90" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A90" s="3"/>
       <c r="B90" s="3"/>
       <c r="C90" s="3"/>
@@ -3177,8 +3468,11 @@
       <c r="X90" s="3"/>
       <c r="Y90" s="3"/>
       <c r="Z90" s="3"/>
-    </row>
-    <row r="91" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA90" s="3"/>
+      <c r="AB90" s="3"/>
+      <c r="AC90" s="3"/>
+    </row>
+    <row r="91" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A91" s="2"/>
       <c r="B91" s="2"/>
       <c r="C91" s="2"/>
@@ -3205,8 +3499,11 @@
       <c r="X91" s="2"/>
       <c r="Y91" s="2"/>
       <c r="Z91" s="2"/>
-    </row>
-    <row r="92" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA91" s="2"/>
+      <c r="AB91" s="2"/>
+      <c r="AC91" s="2"/>
+    </row>
+    <row r="92" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A92" s="3"/>
       <c r="B92" s="3"/>
       <c r="C92" s="3"/>
@@ -3233,8 +3530,11 @@
       <c r="X92" s="3"/>
       <c r="Y92" s="3"/>
       <c r="Z92" s="3"/>
-    </row>
-    <row r="93" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA92" s="3"/>
+      <c r="AB92" s="3"/>
+      <c r="AC92" s="3"/>
+    </row>
+    <row r="93" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A93" s="2"/>
       <c r="B93" s="2"/>
       <c r="C93" s="2"/>
@@ -3261,8 +3561,11 @@
       <c r="X93" s="2"/>
       <c r="Y93" s="2"/>
       <c r="Z93" s="2"/>
-    </row>
-    <row r="94" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA93" s="2"/>
+      <c r="AB93" s="2"/>
+      <c r="AC93" s="2"/>
+    </row>
+    <row r="94" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A94" s="3"/>
       <c r="B94" s="3"/>
       <c r="C94" s="3"/>
@@ -3289,8 +3592,11 @@
       <c r="X94" s="3"/>
       <c r="Y94" s="3"/>
       <c r="Z94" s="3"/>
-    </row>
-    <row r="95" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA94" s="3"/>
+      <c r="AB94" s="3"/>
+      <c r="AC94" s="3"/>
+    </row>
+    <row r="95" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A95" s="2"/>
       <c r="B95" s="2"/>
       <c r="C95" s="2"/>
@@ -3317,8 +3623,11 @@
       <c r="X95" s="2"/>
       <c r="Y95" s="2"/>
       <c r="Z95" s="2"/>
-    </row>
-    <row r="96" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA95" s="2"/>
+      <c r="AB95" s="2"/>
+      <c r="AC95" s="2"/>
+    </row>
+    <row r="96" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A96" s="3"/>
       <c r="B96" s="3"/>
       <c r="C96" s="3"/>
@@ -3345,8 +3654,11 @@
       <c r="X96" s="3"/>
       <c r="Y96" s="3"/>
       <c r="Z96" s="3"/>
-    </row>
-    <row r="97" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA96" s="3"/>
+      <c r="AB96" s="3"/>
+      <c r="AC96" s="3"/>
+    </row>
+    <row r="97" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A97" s="2"/>
       <c r="B97" s="2"/>
       <c r="C97" s="2"/>
@@ -3373,8 +3685,11 @@
       <c r="X97" s="2"/>
       <c r="Y97" s="2"/>
       <c r="Z97" s="2"/>
-    </row>
-    <row r="98" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA97" s="2"/>
+      <c r="AB97" s="2"/>
+      <c r="AC97" s="2"/>
+    </row>
+    <row r="98" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A98" s="3"/>
       <c r="B98" s="3"/>
       <c r="C98" s="3"/>
@@ -3401,8 +3716,11 @@
       <c r="X98" s="3"/>
       <c r="Y98" s="3"/>
       <c r="Z98" s="3"/>
-    </row>
-    <row r="99" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA98" s="3"/>
+      <c r="AB98" s="3"/>
+      <c r="AC98" s="3"/>
+    </row>
+    <row r="99" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A99" s="2"/>
       <c r="B99" s="2"/>
       <c r="C99" s="2"/>
@@ -3429,8 +3747,11 @@
       <c r="X99" s="2"/>
       <c r="Y99" s="2"/>
       <c r="Z99" s="2"/>
-    </row>
-    <row r="100" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AA99" s="2"/>
+      <c r="AB99" s="2"/>
+      <c r="AC99" s="2"/>
+    </row>
+    <row r="100" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A100" s="3"/>
       <c r="B100" s="3"/>
       <c r="C100" s="3"/>
@@ -3457,10 +3778,13 @@
       <c r="X100" s="3"/>
       <c r="Y100" s="3"/>
       <c r="Z100" s="3"/>
+      <c r="AA100" s="3"/>
+      <c r="AB100" s="3"/>
+      <c r="AC100" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:Z1"/>
+    <mergeCell ref="A1:AC1"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat: Add 30 and 90 days to Tenable global metrics export
</commit_message>
<xml_diff>
--- a/client/src/assets/CPAT_METRICS_TEMPLATE.xlsx
+++ b/client/src/assets/CPAT_METRICS_TEMPLATE.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30404"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\C-PAT\client\src\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C5E5DE7-587E-486C-9200-8B5AC937B5D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="39" documentId="13_ncr:1_{6C5E5DE7-587E-486C-9200-8B5AC937B5D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{81CBC0D7-89AB-46F2-BFA0-A61323DEC842}"/>
   <bookViews>
     <workbookView xWindow="24560" yWindow="1760" windowWidth="48060" windowHeight="18060" xr2:uid="{FE1367BE-B521-41BF-8347-968009F83E3B}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +39,13 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+  <si>
+    <t>***** UNCLASSIFIED *****</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Collection </t>
+  </si>
   <si>
     <t xml:space="preserve">Year </t>
   </si>
@@ -68,16 +74,58 @@
     <t>eMASS H/W List - # of Deep Storage Assets</t>
   </si>
   <si>
+    <t>Collection Type</t>
+  </si>
+  <si>
+    <t>Asset Quantity</t>
+  </si>
+  <si>
     <t>Inventory - ACAS Asset Coverage %</t>
   </si>
   <si>
     <t>Inventory - STIGMAN Asset Coverage %</t>
   </si>
   <si>
-    <t>Collection Type</t>
+    <t xml:space="preserve">ACAS Vulnerability Per Host (VPH) Score </t>
   </si>
   <si>
-    <t xml:space="preserve">Collection </t>
+    <t>ACAS Security End of Life Software Findings</t>
+  </si>
+  <si>
+    <t>STIG Compliance CORA Risk Score</t>
+  </si>
+  <si>
+    <t>POAM Coverage (STIGs) % CAT I (High/Criticals)</t>
+  </si>
+  <si>
+    <t>POAM Coverage (STIGs) % CAT II (Mediums)</t>
+  </si>
+  <si>
+    <t>Open Findings CAT I (Total)</t>
+  </si>
+  <si>
+    <t>Open Findings CAT II (Total)</t>
+  </si>
+  <si>
+    <t>Open Findings CAT III (Total)</t>
+  </si>
+  <si>
+    <t>Open Findings (ACAS) CAT I (Within 30 Days)</t>
+  </si>
+  <si>
+    <t>Open Findings (ACAS) CAT II (Within 30 Days)</t>
+  </si>
+  <si>
+    <t>Open Findings (ACAS) CAT III (Within 30 Days)</t>
+  </si>
+  <si>
+    <t>Open Findings (ACAS) CAT I (Within 90 Days)</t>
+  </si>
+  <si>
+    <t>Open Findings (ACAS) CAT II (Within 90 Days)</t>
+  </si>
+  <si>
+    <t>Open Findings (ACAS) CAT III (Within 90 Days)</t>
   </si>
   <si>
     <t>POAM Coverage (ACAS) % CAT I 30+ Days</t>
@@ -89,30 +137,6 @@
     <t>POAM Coverage (ACAS) % CAT III 30+ Days</t>
   </si>
   <si>
-    <t>POAM Coverage (STIGs) % CAT I (High/Criticals)</t>
-  </si>
-  <si>
-    <t>POAM Coverage (STIGs) % CAT II (Mediums)</t>
-  </si>
-  <si>
-    <t>POAM Coverage (STIGs) % CAT III (Lows)</t>
-  </si>
-  <si>
-    <t>STIG Compliance CORA Risk Score</t>
-  </si>
-  <si>
-    <t>ACAS Security End of Life Software Findings</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ACAS Vulnerability Per Host (VPH) Score </t>
-  </si>
-  <si>
-    <t>Asset Quantity</t>
-  </si>
-  <si>
-    <t>***** UNCLASSIFIED *****</t>
-  </si>
-  <si>
     <t>POAM Coverage (ACAS) % CAT I 90+ Days</t>
   </si>
   <si>
@@ -122,20 +146,14 @@
     <t>POAM Coverage (ACAS) % CAT III 90+ Days</t>
   </si>
   <si>
-    <t>Open Findings CAT I (Total)</t>
-  </si>
-  <si>
-    <t>Open Findings CAT II (Total)</t>
-  </si>
-  <si>
-    <t>Open Findings CAT III (Total)</t>
+    <t>POAM Coverage (STIGs) % CAT III (Lows)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -247,7 +265,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -259,6 +277,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -601,30 +622,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FC4E6CA-B04F-4BFD-ADE5-E64E7B1F6F62}">
-  <dimension ref="A1:AC100"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:AI100"/>
+  <sheetFormatPr defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="21.453125" customWidth="1"/>
-    <col min="3" max="3" width="15.90625" customWidth="1"/>
-    <col min="4" max="4" width="10.26953125" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="12.1796875" hidden="1" customWidth="1"/>
-    <col min="6" max="6" width="21.90625" hidden="1" customWidth="1"/>
-    <col min="7" max="7" width="28.6328125" hidden="1" customWidth="1"/>
-    <col min="8" max="8" width="16.54296875" hidden="1" customWidth="1"/>
-    <col min="9" max="9" width="17.36328125" hidden="1" customWidth="1"/>
-    <col min="10" max="10" width="43.90625" hidden="1" customWidth="1"/>
-    <col min="11" max="11" width="14.81640625" customWidth="1"/>
-    <col min="13" max="13" width="14.6328125" hidden="1" customWidth="1"/>
-    <col min="14" max="14" width="12.7265625" hidden="1" customWidth="1"/>
-    <col min="15" max="16" width="19.54296875" customWidth="1"/>
-    <col min="17" max="17" width="16.81640625" customWidth="1"/>
-    <col min="18" max="23" width="25.6328125" customWidth="1"/>
-    <col min="24" max="29" width="23.1796875" customWidth="1"/>
+    <col min="1" max="1" width="21.42578125" customWidth="1"/>
+    <col min="3" max="3" width="15.85546875" customWidth="1"/>
+    <col min="4" max="4" width="10.28515625" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="12.140625" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="21.85546875" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="28.5703125" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="16.5703125" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="17.42578125" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="43.85546875" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="14.85546875" customWidth="1"/>
+    <col min="13" max="13" width="14.5703125" hidden="1" customWidth="1"/>
+    <col min="14" max="14" width="12.7109375" hidden="1" customWidth="1"/>
+    <col min="15" max="16" width="19.5703125" customWidth="1"/>
+    <col min="17" max="17" width="16.85546875" customWidth="1"/>
+    <col min="18" max="26" width="25.5703125" customWidth="1"/>
+    <col min="27" max="35" width="23.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" ht="18.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" ht="18.600000000000001" customHeight="1">
       <c r="A1" s="4" t="s">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
@@ -654,97 +675,121 @@
       <c r="AA1" s="4"/>
       <c r="AB1" s="4"/>
       <c r="AC1" s="4"/>
-    </row>
-    <row r="2" spans="1:29" ht="67.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD1" s="4"/>
+      <c r="AE1" s="4"/>
+      <c r="AF1" s="4"/>
+      <c r="AG1" s="4"/>
+      <c r="AH1" s="4"/>
+      <c r="AI1" s="4"/>
+    </row>
+    <row r="2" spans="1:35" ht="67.5" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K2" s="1" t="s">
         <v>11</v>
       </c>
       <c r="L2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="R2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="S2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="U2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W2" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="M2" s="1" t="s">
-        <v>9</v>
+      <c r="X2" s="1" t="s">
+        <v>23</v>
       </c>
-      <c r="N2" s="1" t="s">
-        <v>10</v>
+      <c r="Y2" s="1" t="s">
+        <v>24</v>
       </c>
-      <c r="O2" s="1" t="s">
-        <v>21</v>
+      <c r="Z2" s="1" t="s">
+        <v>25</v>
       </c>
-      <c r="P2" s="1" t="s">
-        <v>20</v>
+      <c r="AA2" s="1" t="s">
+        <v>26</v>
       </c>
-      <c r="Q2" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="R2" s="1" t="s">
+      <c r="AB2" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="S2" s="1" t="s">
+      <c r="AC2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="T2" s="1" t="s">
+      <c r="AD2" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="U2" s="1" t="s">
-        <v>13</v>
+      <c r="AE2" s="1" t="s">
+        <v>30</v>
       </c>
-      <c r="V2" s="1" t="s">
-        <v>14</v>
+      <c r="AF2" s="1" t="s">
+        <v>31</v>
       </c>
-      <c r="W2" s="1" t="s">
-        <v>15</v>
+      <c r="AG2" s="1" t="s">
+        <v>32</v>
       </c>
-      <c r="X2" s="1" t="s">
-        <v>24</v>
+      <c r="AH2" s="1" t="s">
+        <v>33</v>
       </c>
-      <c r="Y2" s="1" t="s">
-        <v>25</v>
+      <c r="AI2" s="1" t="s">
+        <v>34</v>
       </c>
-      <c r="Z2" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="AA2" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="AB2" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="AC2" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="3" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="3" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -774,8 +819,14 @@
       <c r="AA3" s="2"/>
       <c r="AB3" s="2"/>
       <c r="AC3" s="2"/>
-    </row>
-    <row r="4" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD3" s="2"/>
+      <c r="AE3" s="2"/>
+      <c r="AF3" s="2"/>
+      <c r="AG3" s="2"/>
+      <c r="AH3" s="2"/>
+      <c r="AI3" s="2"/>
+    </row>
+    <row r="4" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A4" s="3"/>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -805,8 +856,14 @@
       <c r="AA4" s="3"/>
       <c r="AB4" s="3"/>
       <c r="AC4" s="3"/>
-    </row>
-    <row r="5" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD4" s="3"/>
+      <c r="AE4" s="3"/>
+      <c r="AF4" s="3"/>
+      <c r="AG4" s="3"/>
+      <c r="AH4" s="3"/>
+      <c r="AI4" s="3"/>
+    </row>
+    <row r="5" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -836,8 +893,14 @@
       <c r="AA5" s="2"/>
       <c r="AB5" s="2"/>
       <c r="AC5" s="2"/>
-    </row>
-    <row r="6" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD5" s="2"/>
+      <c r="AE5" s="2"/>
+      <c r="AF5" s="2"/>
+      <c r="AG5" s="2"/>
+      <c r="AH5" s="2"/>
+      <c r="AI5" s="2"/>
+    </row>
+    <row r="6" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
@@ -867,8 +930,14 @@
       <c r="AA6" s="3"/>
       <c r="AB6" s="3"/>
       <c r="AC6" s="3"/>
-    </row>
-    <row r="7" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD6" s="3"/>
+      <c r="AE6" s="3"/>
+      <c r="AF6" s="3"/>
+      <c r="AG6" s="3"/>
+      <c r="AH6" s="3"/>
+      <c r="AI6" s="3"/>
+    </row>
+    <row r="7" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -898,8 +967,14 @@
       <c r="AA7" s="2"/>
       <c r="AB7" s="2"/>
       <c r="AC7" s="2"/>
-    </row>
-    <row r="8" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD7" s="2"/>
+      <c r="AE7" s="2"/>
+      <c r="AF7" s="2"/>
+      <c r="AG7" s="2"/>
+      <c r="AH7" s="2"/>
+      <c r="AI7" s="2"/>
+    </row>
+    <row r="8" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A8" s="3"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
@@ -929,8 +1004,14 @@
       <c r="AA8" s="3"/>
       <c r="AB8" s="3"/>
       <c r="AC8" s="3"/>
-    </row>
-    <row r="9" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD8" s="3"/>
+      <c r="AE8" s="3"/>
+      <c r="AF8" s="3"/>
+      <c r="AG8" s="3"/>
+      <c r="AH8" s="3"/>
+      <c r="AI8" s="3"/>
+    </row>
+    <row r="9" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="C9" s="2"/>
@@ -960,8 +1041,14 @@
       <c r="AA9" s="2"/>
       <c r="AB9" s="2"/>
       <c r="AC9" s="2"/>
-    </row>
-    <row r="10" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD9" s="2"/>
+      <c r="AE9" s="2"/>
+      <c r="AF9" s="2"/>
+      <c r="AG9" s="2"/>
+      <c r="AH9" s="2"/>
+      <c r="AI9" s="2"/>
+    </row>
+    <row r="10" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A10" s="3"/>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
@@ -991,8 +1078,14 @@
       <c r="AA10" s="3"/>
       <c r="AB10" s="3"/>
       <c r="AC10" s="3"/>
-    </row>
-    <row r="11" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD10" s="3"/>
+      <c r="AE10" s="3"/>
+      <c r="AF10" s="3"/>
+      <c r="AG10" s="3"/>
+      <c r="AH10" s="3"/>
+      <c r="AI10" s="3"/>
+    </row>
+    <row r="11" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -1022,8 +1115,14 @@
       <c r="AA11" s="2"/>
       <c r="AB11" s="2"/>
       <c r="AC11" s="2"/>
-    </row>
-    <row r="12" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD11" s="2"/>
+      <c r="AE11" s="2"/>
+      <c r="AF11" s="2"/>
+      <c r="AG11" s="2"/>
+      <c r="AH11" s="2"/>
+      <c r="AI11" s="2"/>
+    </row>
+    <row r="12" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A12" s="3"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
@@ -1053,8 +1152,14 @@
       <c r="AA12" s="3"/>
       <c r="AB12" s="3"/>
       <c r="AC12" s="3"/>
-    </row>
-    <row r="13" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD12" s="3"/>
+      <c r="AE12" s="3"/>
+      <c r="AF12" s="3"/>
+      <c r="AG12" s="3"/>
+      <c r="AH12" s="3"/>
+      <c r="AI12" s="3"/>
+    </row>
+    <row r="13" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -1084,8 +1189,14 @@
       <c r="AA13" s="2"/>
       <c r="AB13" s="2"/>
       <c r="AC13" s="2"/>
-    </row>
-    <row r="14" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD13" s="2"/>
+      <c r="AE13" s="2"/>
+      <c r="AF13" s="2"/>
+      <c r="AG13" s="2"/>
+      <c r="AH13" s="2"/>
+      <c r="AI13" s="2"/>
+    </row>
+    <row r="14" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A14" s="3"/>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
@@ -1115,8 +1226,14 @@
       <c r="AA14" s="3"/>
       <c r="AB14" s="3"/>
       <c r="AC14" s="3"/>
-    </row>
-    <row r="15" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD14" s="3"/>
+      <c r="AE14" s="3"/>
+      <c r="AF14" s="3"/>
+      <c r="AG14" s="3"/>
+      <c r="AH14" s="3"/>
+      <c r="AI14" s="3"/>
+    </row>
+    <row r="15" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -1146,8 +1263,14 @@
       <c r="AA15" s="2"/>
       <c r="AB15" s="2"/>
       <c r="AC15" s="2"/>
-    </row>
-    <row r="16" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD15" s="2"/>
+      <c r="AE15" s="2"/>
+      <c r="AF15" s="2"/>
+      <c r="AG15" s="2"/>
+      <c r="AH15" s="2"/>
+      <c r="AI15" s="2"/>
+    </row>
+    <row r="16" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A16" s="3"/>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
@@ -1177,8 +1300,14 @@
       <c r="AA16" s="3"/>
       <c r="AB16" s="3"/>
       <c r="AC16" s="3"/>
-    </row>
-    <row r="17" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD16" s="3"/>
+      <c r="AE16" s="3"/>
+      <c r="AF16" s="3"/>
+      <c r="AG16" s="3"/>
+      <c r="AH16" s="3"/>
+      <c r="AI16" s="3"/>
+    </row>
+    <row r="17" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -1208,8 +1337,14 @@
       <c r="AA17" s="2"/>
       <c r="AB17" s="2"/>
       <c r="AC17" s="2"/>
-    </row>
-    <row r="18" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD17" s="2"/>
+      <c r="AE17" s="2"/>
+      <c r="AF17" s="2"/>
+      <c r="AG17" s="2"/>
+      <c r="AH17" s="2"/>
+      <c r="AI17" s="2"/>
+    </row>
+    <row r="18" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A18" s="3"/>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
@@ -1239,8 +1374,14 @@
       <c r="AA18" s="3"/>
       <c r="AB18" s="3"/>
       <c r="AC18" s="3"/>
-    </row>
-    <row r="19" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD18" s="3"/>
+      <c r="AE18" s="3"/>
+      <c r="AF18" s="3"/>
+      <c r="AG18" s="3"/>
+      <c r="AH18" s="3"/>
+      <c r="AI18" s="3"/>
+    </row>
+    <row r="19" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -1270,8 +1411,14 @@
       <c r="AA19" s="2"/>
       <c r="AB19" s="2"/>
       <c r="AC19" s="2"/>
-    </row>
-    <row r="20" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD19" s="2"/>
+      <c r="AE19" s="2"/>
+      <c r="AF19" s="2"/>
+      <c r="AG19" s="2"/>
+      <c r="AH19" s="2"/>
+      <c r="AI19" s="2"/>
+    </row>
+    <row r="20" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A20" s="3"/>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
@@ -1301,8 +1448,14 @@
       <c r="AA20" s="3"/>
       <c r="AB20" s="3"/>
       <c r="AC20" s="3"/>
-    </row>
-    <row r="21" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD20" s="3"/>
+      <c r="AE20" s="3"/>
+      <c r="AF20" s="3"/>
+      <c r="AG20" s="3"/>
+      <c r="AH20" s="3"/>
+      <c r="AI20" s="3"/>
+    </row>
+    <row r="21" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -1332,8 +1485,14 @@
       <c r="AA21" s="2"/>
       <c r="AB21" s="2"/>
       <c r="AC21" s="2"/>
-    </row>
-    <row r="22" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD21" s="2"/>
+      <c r="AE21" s="2"/>
+      <c r="AF21" s="2"/>
+      <c r="AG21" s="2"/>
+      <c r="AH21" s="2"/>
+      <c r="AI21" s="2"/>
+    </row>
+    <row r="22" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A22" s="3"/>
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
@@ -1363,8 +1522,14 @@
       <c r="AA22" s="3"/>
       <c r="AB22" s="3"/>
       <c r="AC22" s="3"/>
-    </row>
-    <row r="23" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD22" s="3"/>
+      <c r="AE22" s="3"/>
+      <c r="AF22" s="3"/>
+      <c r="AG22" s="3"/>
+      <c r="AH22" s="3"/>
+      <c r="AI22" s="3"/>
+    </row>
+    <row r="23" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
@@ -1394,8 +1559,14 @@
       <c r="AA23" s="2"/>
       <c r="AB23" s="2"/>
       <c r="AC23" s="2"/>
-    </row>
-    <row r="24" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD23" s="2"/>
+      <c r="AE23" s="2"/>
+      <c r="AF23" s="2"/>
+      <c r="AG23" s="2"/>
+      <c r="AH23" s="2"/>
+      <c r="AI23" s="2"/>
+    </row>
+    <row r="24" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A24" s="3"/>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
@@ -1425,8 +1596,14 @@
       <c r="AA24" s="3"/>
       <c r="AB24" s="3"/>
       <c r="AC24" s="3"/>
-    </row>
-    <row r="25" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD24" s="3"/>
+      <c r="AE24" s="3"/>
+      <c r="AF24" s="3"/>
+      <c r="AG24" s="3"/>
+      <c r="AH24" s="3"/>
+      <c r="AI24" s="3"/>
+    </row>
+    <row r="25" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
@@ -1456,8 +1633,14 @@
       <c r="AA25" s="2"/>
       <c r="AB25" s="2"/>
       <c r="AC25" s="2"/>
-    </row>
-    <row r="26" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD25" s="2"/>
+      <c r="AE25" s="2"/>
+      <c r="AF25" s="2"/>
+      <c r="AG25" s="2"/>
+      <c r="AH25" s="2"/>
+      <c r="AI25" s="2"/>
+    </row>
+    <row r="26" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A26" s="3"/>
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
@@ -1487,8 +1670,14 @@
       <c r="AA26" s="3"/>
       <c r="AB26" s="3"/>
       <c r="AC26" s="3"/>
-    </row>
-    <row r="27" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD26" s="3"/>
+      <c r="AE26" s="3"/>
+      <c r="AF26" s="3"/>
+      <c r="AG26" s="3"/>
+      <c r="AH26" s="3"/>
+      <c r="AI26" s="3"/>
+    </row>
+    <row r="27" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
@@ -1518,8 +1707,14 @@
       <c r="AA27" s="2"/>
       <c r="AB27" s="2"/>
       <c r="AC27" s="2"/>
-    </row>
-    <row r="28" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD27" s="2"/>
+      <c r="AE27" s="2"/>
+      <c r="AF27" s="2"/>
+      <c r="AG27" s="2"/>
+      <c r="AH27" s="2"/>
+      <c r="AI27" s="2"/>
+    </row>
+    <row r="28" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A28" s="3"/>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
@@ -1549,8 +1744,14 @@
       <c r="AA28" s="3"/>
       <c r="AB28" s="3"/>
       <c r="AC28" s="3"/>
-    </row>
-    <row r="29" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD28" s="3"/>
+      <c r="AE28" s="3"/>
+      <c r="AF28" s="3"/>
+      <c r="AG28" s="3"/>
+      <c r="AH28" s="3"/>
+      <c r="AI28" s="3"/>
+    </row>
+    <row r="29" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
@@ -1580,8 +1781,14 @@
       <c r="AA29" s="2"/>
       <c r="AB29" s="2"/>
       <c r="AC29" s="2"/>
-    </row>
-    <row r="30" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD29" s="2"/>
+      <c r="AE29" s="2"/>
+      <c r="AF29" s="2"/>
+      <c r="AG29" s="2"/>
+      <c r="AH29" s="2"/>
+      <c r="AI29" s="2"/>
+    </row>
+    <row r="30" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A30" s="3"/>
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
@@ -1611,8 +1818,14 @@
       <c r="AA30" s="3"/>
       <c r="AB30" s="3"/>
       <c r="AC30" s="3"/>
-    </row>
-    <row r="31" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD30" s="3"/>
+      <c r="AE30" s="3"/>
+      <c r="AF30" s="3"/>
+      <c r="AG30" s="3"/>
+      <c r="AH30" s="3"/>
+      <c r="AI30" s="3"/>
+    </row>
+    <row r="31" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
@@ -1642,8 +1855,14 @@
       <c r="AA31" s="2"/>
       <c r="AB31" s="2"/>
       <c r="AC31" s="2"/>
-    </row>
-    <row r="32" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD31" s="2"/>
+      <c r="AE31" s="2"/>
+      <c r="AF31" s="2"/>
+      <c r="AG31" s="2"/>
+      <c r="AH31" s="2"/>
+      <c r="AI31" s="2"/>
+    </row>
+    <row r="32" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A32" s="3"/>
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
@@ -1673,8 +1892,14 @@
       <c r="AA32" s="3"/>
       <c r="AB32" s="3"/>
       <c r="AC32" s="3"/>
-    </row>
-    <row r="33" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD32" s="3"/>
+      <c r="AE32" s="3"/>
+      <c r="AF32" s="3"/>
+      <c r="AG32" s="3"/>
+      <c r="AH32" s="3"/>
+      <c r="AI32" s="3"/>
+    </row>
+    <row r="33" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
@@ -1704,8 +1929,14 @@
       <c r="AA33" s="2"/>
       <c r="AB33" s="2"/>
       <c r="AC33" s="2"/>
-    </row>
-    <row r="34" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD33" s="2"/>
+      <c r="AE33" s="2"/>
+      <c r="AF33" s="2"/>
+      <c r="AG33" s="2"/>
+      <c r="AH33" s="2"/>
+      <c r="AI33" s="2"/>
+    </row>
+    <row r="34" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A34" s="3"/>
       <c r="B34" s="3"/>
       <c r="C34" s="3"/>
@@ -1735,8 +1966,14 @@
       <c r="AA34" s="3"/>
       <c r="AB34" s="3"/>
       <c r="AC34" s="3"/>
-    </row>
-    <row r="35" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD34" s="3"/>
+      <c r="AE34" s="3"/>
+      <c r="AF34" s="3"/>
+      <c r="AG34" s="3"/>
+      <c r="AH34" s="3"/>
+      <c r="AI34" s="3"/>
+    </row>
+    <row r="35" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A35" s="2"/>
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
@@ -1766,8 +2003,14 @@
       <c r="AA35" s="2"/>
       <c r="AB35" s="2"/>
       <c r="AC35" s="2"/>
-    </row>
-    <row r="36" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD35" s="2"/>
+      <c r="AE35" s="2"/>
+      <c r="AF35" s="2"/>
+      <c r="AG35" s="2"/>
+      <c r="AH35" s="2"/>
+      <c r="AI35" s="2"/>
+    </row>
+    <row r="36" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A36" s="3"/>
       <c r="B36" s="3"/>
       <c r="C36" s="3"/>
@@ -1797,8 +2040,14 @@
       <c r="AA36" s="3"/>
       <c r="AB36" s="3"/>
       <c r="AC36" s="3"/>
-    </row>
-    <row r="37" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD36" s="3"/>
+      <c r="AE36" s="3"/>
+      <c r="AF36" s="3"/>
+      <c r="AG36" s="3"/>
+      <c r="AH36" s="3"/>
+      <c r="AI36" s="3"/>
+    </row>
+    <row r="37" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
@@ -1828,8 +2077,14 @@
       <c r="AA37" s="2"/>
       <c r="AB37" s="2"/>
       <c r="AC37" s="2"/>
-    </row>
-    <row r="38" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD37" s="2"/>
+      <c r="AE37" s="2"/>
+      <c r="AF37" s="2"/>
+      <c r="AG37" s="2"/>
+      <c r="AH37" s="2"/>
+      <c r="AI37" s="2"/>
+    </row>
+    <row r="38" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A38" s="3"/>
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
@@ -1859,8 +2114,14 @@
       <c r="AA38" s="3"/>
       <c r="AB38" s="3"/>
       <c r="AC38" s="3"/>
-    </row>
-    <row r="39" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD38" s="3"/>
+      <c r="AE38" s="3"/>
+      <c r="AF38" s="3"/>
+      <c r="AG38" s="3"/>
+      <c r="AH38" s="3"/>
+      <c r="AI38" s="3"/>
+    </row>
+    <row r="39" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A39" s="2"/>
       <c r="B39" s="2"/>
       <c r="C39" s="2"/>
@@ -1890,8 +2151,14 @@
       <c r="AA39" s="2"/>
       <c r="AB39" s="2"/>
       <c r="AC39" s="2"/>
-    </row>
-    <row r="40" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD39" s="2"/>
+      <c r="AE39" s="2"/>
+      <c r="AF39" s="2"/>
+      <c r="AG39" s="2"/>
+      <c r="AH39" s="2"/>
+      <c r="AI39" s="2"/>
+    </row>
+    <row r="40" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A40" s="3"/>
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
@@ -1921,8 +2188,14 @@
       <c r="AA40" s="3"/>
       <c r="AB40" s="3"/>
       <c r="AC40" s="3"/>
-    </row>
-    <row r="41" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD40" s="3"/>
+      <c r="AE40" s="3"/>
+      <c r="AF40" s="3"/>
+      <c r="AG40" s="3"/>
+      <c r="AH40" s="3"/>
+      <c r="AI40" s="3"/>
+    </row>
+    <row r="41" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A41" s="2"/>
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
@@ -1952,8 +2225,14 @@
       <c r="AA41" s="2"/>
       <c r="AB41" s="2"/>
       <c r="AC41" s="2"/>
-    </row>
-    <row r="42" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD41" s="2"/>
+      <c r="AE41" s="2"/>
+      <c r="AF41" s="2"/>
+      <c r="AG41" s="2"/>
+      <c r="AH41" s="2"/>
+      <c r="AI41" s="2"/>
+    </row>
+    <row r="42" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A42" s="3"/>
       <c r="B42" s="3"/>
       <c r="C42" s="3"/>
@@ -1983,8 +2262,14 @@
       <c r="AA42" s="3"/>
       <c r="AB42" s="3"/>
       <c r="AC42" s="3"/>
-    </row>
-    <row r="43" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD42" s="3"/>
+      <c r="AE42" s="3"/>
+      <c r="AF42" s="3"/>
+      <c r="AG42" s="3"/>
+      <c r="AH42" s="3"/>
+      <c r="AI42" s="3"/>
+    </row>
+    <row r="43" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A43" s="2"/>
       <c r="B43" s="2"/>
       <c r="C43" s="2"/>
@@ -2014,8 +2299,14 @@
       <c r="AA43" s="2"/>
       <c r="AB43" s="2"/>
       <c r="AC43" s="2"/>
-    </row>
-    <row r="44" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD43" s="2"/>
+      <c r="AE43" s="2"/>
+      <c r="AF43" s="2"/>
+      <c r="AG43" s="2"/>
+      <c r="AH43" s="2"/>
+      <c r="AI43" s="2"/>
+    </row>
+    <row r="44" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A44" s="3"/>
       <c r="B44" s="3"/>
       <c r="C44" s="3"/>
@@ -2045,8 +2336,14 @@
       <c r="AA44" s="3"/>
       <c r="AB44" s="3"/>
       <c r="AC44" s="3"/>
-    </row>
-    <row r="45" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD44" s="3"/>
+      <c r="AE44" s="3"/>
+      <c r="AF44" s="3"/>
+      <c r="AG44" s="3"/>
+      <c r="AH44" s="3"/>
+      <c r="AI44" s="3"/>
+    </row>
+    <row r="45" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A45" s="2"/>
       <c r="B45" s="2"/>
       <c r="C45" s="2"/>
@@ -2076,8 +2373,14 @@
       <c r="AA45" s="2"/>
       <c r="AB45" s="2"/>
       <c r="AC45" s="2"/>
-    </row>
-    <row r="46" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD45" s="2"/>
+      <c r="AE45" s="2"/>
+      <c r="AF45" s="2"/>
+      <c r="AG45" s="2"/>
+      <c r="AH45" s="2"/>
+      <c r="AI45" s="2"/>
+    </row>
+    <row r="46" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A46" s="3"/>
       <c r="B46" s="3"/>
       <c r="C46" s="3"/>
@@ -2107,8 +2410,14 @@
       <c r="AA46" s="3"/>
       <c r="AB46" s="3"/>
       <c r="AC46" s="3"/>
-    </row>
-    <row r="47" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD46" s="3"/>
+      <c r="AE46" s="3"/>
+      <c r="AF46" s="3"/>
+      <c r="AG46" s="3"/>
+      <c r="AH46" s="3"/>
+      <c r="AI46" s="3"/>
+    </row>
+    <row r="47" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A47" s="2"/>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
@@ -2138,8 +2447,14 @@
       <c r="AA47" s="2"/>
       <c r="AB47" s="2"/>
       <c r="AC47" s="2"/>
-    </row>
-    <row r="48" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD47" s="2"/>
+      <c r="AE47" s="2"/>
+      <c r="AF47" s="2"/>
+      <c r="AG47" s="2"/>
+      <c r="AH47" s="2"/>
+      <c r="AI47" s="2"/>
+    </row>
+    <row r="48" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A48" s="3"/>
       <c r="B48" s="3"/>
       <c r="C48" s="3"/>
@@ -2169,8 +2484,14 @@
       <c r="AA48" s="3"/>
       <c r="AB48" s="3"/>
       <c r="AC48" s="3"/>
-    </row>
-    <row r="49" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD48" s="3"/>
+      <c r="AE48" s="3"/>
+      <c r="AF48" s="3"/>
+      <c r="AG48" s="3"/>
+      <c r="AH48" s="3"/>
+      <c r="AI48" s="3"/>
+    </row>
+    <row r="49" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A49" s="2"/>
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
@@ -2200,8 +2521,14 @@
       <c r="AA49" s="2"/>
       <c r="AB49" s="2"/>
       <c r="AC49" s="2"/>
-    </row>
-    <row r="50" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD49" s="2"/>
+      <c r="AE49" s="2"/>
+      <c r="AF49" s="2"/>
+      <c r="AG49" s="2"/>
+      <c r="AH49" s="2"/>
+      <c r="AI49" s="2"/>
+    </row>
+    <row r="50" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A50" s="3"/>
       <c r="B50" s="3"/>
       <c r="C50" s="3"/>
@@ -2231,8 +2558,14 @@
       <c r="AA50" s="3"/>
       <c r="AB50" s="3"/>
       <c r="AC50" s="3"/>
-    </row>
-    <row r="51" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD50" s="3"/>
+      <c r="AE50" s="3"/>
+      <c r="AF50" s="3"/>
+      <c r="AG50" s="3"/>
+      <c r="AH50" s="3"/>
+      <c r="AI50" s="3"/>
+    </row>
+    <row r="51" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A51" s="2"/>
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
@@ -2262,8 +2595,14 @@
       <c r="AA51" s="2"/>
       <c r="AB51" s="2"/>
       <c r="AC51" s="2"/>
-    </row>
-    <row r="52" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD51" s="2"/>
+      <c r="AE51" s="2"/>
+      <c r="AF51" s="2"/>
+      <c r="AG51" s="2"/>
+      <c r="AH51" s="2"/>
+      <c r="AI51" s="2"/>
+    </row>
+    <row r="52" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A52" s="3"/>
       <c r="B52" s="3"/>
       <c r="C52" s="3"/>
@@ -2293,8 +2632,14 @@
       <c r="AA52" s="3"/>
       <c r="AB52" s="3"/>
       <c r="AC52" s="3"/>
-    </row>
-    <row r="53" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD52" s="3"/>
+      <c r="AE52" s="3"/>
+      <c r="AF52" s="3"/>
+      <c r="AG52" s="3"/>
+      <c r="AH52" s="3"/>
+      <c r="AI52" s="3"/>
+    </row>
+    <row r="53" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A53" s="2"/>
       <c r="B53" s="2"/>
       <c r="C53" s="2"/>
@@ -2324,8 +2669,14 @@
       <c r="AA53" s="2"/>
       <c r="AB53" s="2"/>
       <c r="AC53" s="2"/>
-    </row>
-    <row r="54" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD53" s="2"/>
+      <c r="AE53" s="2"/>
+      <c r="AF53" s="2"/>
+      <c r="AG53" s="2"/>
+      <c r="AH53" s="2"/>
+      <c r="AI53" s="2"/>
+    </row>
+    <row r="54" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A54" s="3"/>
       <c r="B54" s="3"/>
       <c r="C54" s="3"/>
@@ -2355,8 +2706,14 @@
       <c r="AA54" s="3"/>
       <c r="AB54" s="3"/>
       <c r="AC54" s="3"/>
-    </row>
-    <row r="55" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD54" s="3"/>
+      <c r="AE54" s="3"/>
+      <c r="AF54" s="3"/>
+      <c r="AG54" s="3"/>
+      <c r="AH54" s="3"/>
+      <c r="AI54" s="3"/>
+    </row>
+    <row r="55" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A55" s="2"/>
       <c r="B55" s="2"/>
       <c r="C55" s="2"/>
@@ -2386,8 +2743,14 @@
       <c r="AA55" s="2"/>
       <c r="AB55" s="2"/>
       <c r="AC55" s="2"/>
-    </row>
-    <row r="56" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD55" s="2"/>
+      <c r="AE55" s="2"/>
+      <c r="AF55" s="2"/>
+      <c r="AG55" s="2"/>
+      <c r="AH55" s="2"/>
+      <c r="AI55" s="2"/>
+    </row>
+    <row r="56" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A56" s="3"/>
       <c r="B56" s="3"/>
       <c r="C56" s="3"/>
@@ -2417,8 +2780,14 @@
       <c r="AA56" s="3"/>
       <c r="AB56" s="3"/>
       <c r="AC56" s="3"/>
-    </row>
-    <row r="57" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD56" s="3"/>
+      <c r="AE56" s="3"/>
+      <c r="AF56" s="3"/>
+      <c r="AG56" s="3"/>
+      <c r="AH56" s="3"/>
+      <c r="AI56" s="3"/>
+    </row>
+    <row r="57" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A57" s="2"/>
       <c r="B57" s="2"/>
       <c r="C57" s="2"/>
@@ -2448,8 +2817,14 @@
       <c r="AA57" s="2"/>
       <c r="AB57" s="2"/>
       <c r="AC57" s="2"/>
-    </row>
-    <row r="58" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD57" s="2"/>
+      <c r="AE57" s="2"/>
+      <c r="AF57" s="2"/>
+      <c r="AG57" s="2"/>
+      <c r="AH57" s="2"/>
+      <c r="AI57" s="2"/>
+    </row>
+    <row r="58" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A58" s="3"/>
       <c r="B58" s="3"/>
       <c r="C58" s="3"/>
@@ -2479,8 +2854,14 @@
       <c r="AA58" s="3"/>
       <c r="AB58" s="3"/>
       <c r="AC58" s="3"/>
-    </row>
-    <row r="59" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD58" s="3"/>
+      <c r="AE58" s="3"/>
+      <c r="AF58" s="3"/>
+      <c r="AG58" s="3"/>
+      <c r="AH58" s="3"/>
+      <c r="AI58" s="3"/>
+    </row>
+    <row r="59" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A59" s="2"/>
       <c r="B59" s="2"/>
       <c r="C59" s="2"/>
@@ -2510,8 +2891,14 @@
       <c r="AA59" s="2"/>
       <c r="AB59" s="2"/>
       <c r="AC59" s="2"/>
-    </row>
-    <row r="60" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD59" s="2"/>
+      <c r="AE59" s="2"/>
+      <c r="AF59" s="2"/>
+      <c r="AG59" s="2"/>
+      <c r="AH59" s="2"/>
+      <c r="AI59" s="2"/>
+    </row>
+    <row r="60" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A60" s="3"/>
       <c r="B60" s="3"/>
       <c r="C60" s="3"/>
@@ -2541,8 +2928,14 @@
       <c r="AA60" s="3"/>
       <c r="AB60" s="3"/>
       <c r="AC60" s="3"/>
-    </row>
-    <row r="61" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD60" s="3"/>
+      <c r="AE60" s="3"/>
+      <c r="AF60" s="3"/>
+      <c r="AG60" s="3"/>
+      <c r="AH60" s="3"/>
+      <c r="AI60" s="3"/>
+    </row>
+    <row r="61" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A61" s="2"/>
       <c r="B61" s="2"/>
       <c r="C61" s="2"/>
@@ -2572,8 +2965,14 @@
       <c r="AA61" s="2"/>
       <c r="AB61" s="2"/>
       <c r="AC61" s="2"/>
-    </row>
-    <row r="62" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD61" s="2"/>
+      <c r="AE61" s="2"/>
+      <c r="AF61" s="2"/>
+      <c r="AG61" s="2"/>
+      <c r="AH61" s="2"/>
+      <c r="AI61" s="2"/>
+    </row>
+    <row r="62" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A62" s="3"/>
       <c r="B62" s="3"/>
       <c r="C62" s="3"/>
@@ -2603,8 +3002,14 @@
       <c r="AA62" s="3"/>
       <c r="AB62" s="3"/>
       <c r="AC62" s="3"/>
-    </row>
-    <row r="63" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD62" s="3"/>
+      <c r="AE62" s="3"/>
+      <c r="AF62" s="3"/>
+      <c r="AG62" s="3"/>
+      <c r="AH62" s="3"/>
+      <c r="AI62" s="3"/>
+    </row>
+    <row r="63" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A63" s="2"/>
       <c r="B63" s="2"/>
       <c r="C63" s="2"/>
@@ -2634,8 +3039,14 @@
       <c r="AA63" s="2"/>
       <c r="AB63" s="2"/>
       <c r="AC63" s="2"/>
-    </row>
-    <row r="64" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD63" s="2"/>
+      <c r="AE63" s="2"/>
+      <c r="AF63" s="2"/>
+      <c r="AG63" s="2"/>
+      <c r="AH63" s="2"/>
+      <c r="AI63" s="2"/>
+    </row>
+    <row r="64" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A64" s="3"/>
       <c r="B64" s="3"/>
       <c r="C64" s="3"/>
@@ -2665,8 +3076,14 @@
       <c r="AA64" s="3"/>
       <c r="AB64" s="3"/>
       <c r="AC64" s="3"/>
-    </row>
-    <row r="65" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD64" s="3"/>
+      <c r="AE64" s="3"/>
+      <c r="AF64" s="3"/>
+      <c r="AG64" s="3"/>
+      <c r="AH64" s="3"/>
+      <c r="AI64" s="3"/>
+    </row>
+    <row r="65" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A65" s="2"/>
       <c r="B65" s="2"/>
       <c r="C65" s="2"/>
@@ -2696,8 +3113,14 @@
       <c r="AA65" s="2"/>
       <c r="AB65" s="2"/>
       <c r="AC65" s="2"/>
-    </row>
-    <row r="66" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD65" s="2"/>
+      <c r="AE65" s="2"/>
+      <c r="AF65" s="2"/>
+      <c r="AG65" s="2"/>
+      <c r="AH65" s="2"/>
+      <c r="AI65" s="2"/>
+    </row>
+    <row r="66" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A66" s="3"/>
       <c r="B66" s="3"/>
       <c r="C66" s="3"/>
@@ -2727,8 +3150,14 @@
       <c r="AA66" s="3"/>
       <c r="AB66" s="3"/>
       <c r="AC66" s="3"/>
-    </row>
-    <row r="67" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD66" s="3"/>
+      <c r="AE66" s="3"/>
+      <c r="AF66" s="3"/>
+      <c r="AG66" s="3"/>
+      <c r="AH66" s="3"/>
+      <c r="AI66" s="3"/>
+    </row>
+    <row r="67" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A67" s="2"/>
       <c r="B67" s="2"/>
       <c r="C67" s="2"/>
@@ -2758,8 +3187,14 @@
       <c r="AA67" s="2"/>
       <c r="AB67" s="2"/>
       <c r="AC67" s="2"/>
-    </row>
-    <row r="68" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD67" s="2"/>
+      <c r="AE67" s="2"/>
+      <c r="AF67" s="2"/>
+      <c r="AG67" s="2"/>
+      <c r="AH67" s="2"/>
+      <c r="AI67" s="2"/>
+    </row>
+    <row r="68" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A68" s="3"/>
       <c r="B68" s="3"/>
       <c r="C68" s="3"/>
@@ -2789,8 +3224,14 @@
       <c r="AA68" s="3"/>
       <c r="AB68" s="3"/>
       <c r="AC68" s="3"/>
-    </row>
-    <row r="69" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD68" s="3"/>
+      <c r="AE68" s="3"/>
+      <c r="AF68" s="3"/>
+      <c r="AG68" s="3"/>
+      <c r="AH68" s="3"/>
+      <c r="AI68" s="3"/>
+    </row>
+    <row r="69" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A69" s="2"/>
       <c r="B69" s="2"/>
       <c r="C69" s="2"/>
@@ -2820,8 +3261,14 @@
       <c r="AA69" s="2"/>
       <c r="AB69" s="2"/>
       <c r="AC69" s="2"/>
-    </row>
-    <row r="70" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD69" s="2"/>
+      <c r="AE69" s="2"/>
+      <c r="AF69" s="2"/>
+      <c r="AG69" s="2"/>
+      <c r="AH69" s="2"/>
+      <c r="AI69" s="2"/>
+    </row>
+    <row r="70" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A70" s="3"/>
       <c r="B70" s="3"/>
       <c r="C70" s="3"/>
@@ -2851,8 +3298,14 @@
       <c r="AA70" s="3"/>
       <c r="AB70" s="3"/>
       <c r="AC70" s="3"/>
-    </row>
-    <row r="71" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD70" s="3"/>
+      <c r="AE70" s="3"/>
+      <c r="AF70" s="3"/>
+      <c r="AG70" s="3"/>
+      <c r="AH70" s="3"/>
+      <c r="AI70" s="3"/>
+    </row>
+    <row r="71" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A71" s="2"/>
       <c r="B71" s="2"/>
       <c r="C71" s="2"/>
@@ -2882,8 +3335,14 @@
       <c r="AA71" s="2"/>
       <c r="AB71" s="2"/>
       <c r="AC71" s="2"/>
-    </row>
-    <row r="72" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD71" s="2"/>
+      <c r="AE71" s="2"/>
+      <c r="AF71" s="2"/>
+      <c r="AG71" s="2"/>
+      <c r="AH71" s="2"/>
+      <c r="AI71" s="2"/>
+    </row>
+    <row r="72" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A72" s="3"/>
       <c r="B72" s="3"/>
       <c r="C72" s="3"/>
@@ -2913,8 +3372,14 @@
       <c r="AA72" s="3"/>
       <c r="AB72" s="3"/>
       <c r="AC72" s="3"/>
-    </row>
-    <row r="73" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD72" s="3"/>
+      <c r="AE72" s="3"/>
+      <c r="AF72" s="3"/>
+      <c r="AG72" s="3"/>
+      <c r="AH72" s="3"/>
+      <c r="AI72" s="3"/>
+    </row>
+    <row r="73" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A73" s="2"/>
       <c r="B73" s="2"/>
       <c r="C73" s="2"/>
@@ -2944,8 +3409,14 @@
       <c r="AA73" s="2"/>
       <c r="AB73" s="2"/>
       <c r="AC73" s="2"/>
-    </row>
-    <row r="74" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD73" s="2"/>
+      <c r="AE73" s="2"/>
+      <c r="AF73" s="2"/>
+      <c r="AG73" s="2"/>
+      <c r="AH73" s="2"/>
+      <c r="AI73" s="2"/>
+    </row>
+    <row r="74" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A74" s="3"/>
       <c r="B74" s="3"/>
       <c r="C74" s="3"/>
@@ -2975,8 +3446,14 @@
       <c r="AA74" s="3"/>
       <c r="AB74" s="3"/>
       <c r="AC74" s="3"/>
-    </row>
-    <row r="75" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD74" s="3"/>
+      <c r="AE74" s="3"/>
+      <c r="AF74" s="3"/>
+      <c r="AG74" s="3"/>
+      <c r="AH74" s="3"/>
+      <c r="AI74" s="3"/>
+    </row>
+    <row r="75" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A75" s="2"/>
       <c r="B75" s="2"/>
       <c r="C75" s="2"/>
@@ -3006,8 +3483,14 @@
       <c r="AA75" s="2"/>
       <c r="AB75" s="2"/>
       <c r="AC75" s="2"/>
-    </row>
-    <row r="76" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD75" s="2"/>
+      <c r="AE75" s="2"/>
+      <c r="AF75" s="2"/>
+      <c r="AG75" s="2"/>
+      <c r="AH75" s="2"/>
+      <c r="AI75" s="2"/>
+    </row>
+    <row r="76" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A76" s="3"/>
       <c r="B76" s="3"/>
       <c r="C76" s="3"/>
@@ -3037,8 +3520,14 @@
       <c r="AA76" s="3"/>
       <c r="AB76" s="3"/>
       <c r="AC76" s="3"/>
-    </row>
-    <row r="77" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD76" s="3"/>
+      <c r="AE76" s="3"/>
+      <c r="AF76" s="3"/>
+      <c r="AG76" s="3"/>
+      <c r="AH76" s="3"/>
+      <c r="AI76" s="3"/>
+    </row>
+    <row r="77" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A77" s="2"/>
       <c r="B77" s="2"/>
       <c r="C77" s="2"/>
@@ -3068,8 +3557,14 @@
       <c r="AA77" s="2"/>
       <c r="AB77" s="2"/>
       <c r="AC77" s="2"/>
-    </row>
-    <row r="78" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD77" s="2"/>
+      <c r="AE77" s="2"/>
+      <c r="AF77" s="2"/>
+      <c r="AG77" s="2"/>
+      <c r="AH77" s="2"/>
+      <c r="AI77" s="2"/>
+    </row>
+    <row r="78" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A78" s="3"/>
       <c r="B78" s="3"/>
       <c r="C78" s="3"/>
@@ -3099,8 +3594,14 @@
       <c r="AA78" s="3"/>
       <c r="AB78" s="3"/>
       <c r="AC78" s="3"/>
-    </row>
-    <row r="79" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD78" s="3"/>
+      <c r="AE78" s="3"/>
+      <c r="AF78" s="3"/>
+      <c r="AG78" s="3"/>
+      <c r="AH78" s="3"/>
+      <c r="AI78" s="3"/>
+    </row>
+    <row r="79" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A79" s="2"/>
       <c r="B79" s="2"/>
       <c r="C79" s="2"/>
@@ -3130,8 +3631,14 @@
       <c r="AA79" s="2"/>
       <c r="AB79" s="2"/>
       <c r="AC79" s="2"/>
-    </row>
-    <row r="80" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD79" s="2"/>
+      <c r="AE79" s="2"/>
+      <c r="AF79" s="2"/>
+      <c r="AG79" s="2"/>
+      <c r="AH79" s="2"/>
+      <c r="AI79" s="2"/>
+    </row>
+    <row r="80" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A80" s="3"/>
       <c r="B80" s="3"/>
       <c r="C80" s="3"/>
@@ -3161,8 +3668,14 @@
       <c r="AA80" s="3"/>
       <c r="AB80" s="3"/>
       <c r="AC80" s="3"/>
-    </row>
-    <row r="81" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD80" s="3"/>
+      <c r="AE80" s="3"/>
+      <c r="AF80" s="3"/>
+      <c r="AG80" s="3"/>
+      <c r="AH80" s="3"/>
+      <c r="AI80" s="3"/>
+    </row>
+    <row r="81" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A81" s="2"/>
       <c r="B81" s="2"/>
       <c r="C81" s="2"/>
@@ -3192,8 +3705,14 @@
       <c r="AA81" s="2"/>
       <c r="AB81" s="2"/>
       <c r="AC81" s="2"/>
-    </row>
-    <row r="82" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD81" s="2"/>
+      <c r="AE81" s="2"/>
+      <c r="AF81" s="2"/>
+      <c r="AG81" s="2"/>
+      <c r="AH81" s="2"/>
+      <c r="AI81" s="2"/>
+    </row>
+    <row r="82" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A82" s="3"/>
       <c r="B82" s="3"/>
       <c r="C82" s="3"/>
@@ -3223,8 +3742,14 @@
       <c r="AA82" s="3"/>
       <c r="AB82" s="3"/>
       <c r="AC82" s="3"/>
-    </row>
-    <row r="83" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD82" s="3"/>
+      <c r="AE82" s="3"/>
+      <c r="AF82" s="3"/>
+      <c r="AG82" s="3"/>
+      <c r="AH82" s="3"/>
+      <c r="AI82" s="3"/>
+    </row>
+    <row r="83" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A83" s="2"/>
       <c r="B83" s="2"/>
       <c r="C83" s="2"/>
@@ -3254,8 +3779,14 @@
       <c r="AA83" s="2"/>
       <c r="AB83" s="2"/>
       <c r="AC83" s="2"/>
-    </row>
-    <row r="84" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD83" s="2"/>
+      <c r="AE83" s="2"/>
+      <c r="AF83" s="2"/>
+      <c r="AG83" s="2"/>
+      <c r="AH83" s="2"/>
+      <c r="AI83" s="2"/>
+    </row>
+    <row r="84" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A84" s="3"/>
       <c r="B84" s="3"/>
       <c r="C84" s="3"/>
@@ -3285,8 +3816,14 @@
       <c r="AA84" s="3"/>
       <c r="AB84" s="3"/>
       <c r="AC84" s="3"/>
-    </row>
-    <row r="85" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD84" s="3"/>
+      <c r="AE84" s="3"/>
+      <c r="AF84" s="3"/>
+      <c r="AG84" s="3"/>
+      <c r="AH84" s="3"/>
+      <c r="AI84" s="3"/>
+    </row>
+    <row r="85" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A85" s="2"/>
       <c r="B85" s="2"/>
       <c r="C85" s="2"/>
@@ -3316,8 +3853,14 @@
       <c r="AA85" s="2"/>
       <c r="AB85" s="2"/>
       <c r="AC85" s="2"/>
-    </row>
-    <row r="86" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD85" s="2"/>
+      <c r="AE85" s="2"/>
+      <c r="AF85" s="2"/>
+      <c r="AG85" s="2"/>
+      <c r="AH85" s="2"/>
+      <c r="AI85" s="2"/>
+    </row>
+    <row r="86" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A86" s="3"/>
       <c r="B86" s="3"/>
       <c r="C86" s="3"/>
@@ -3347,8 +3890,14 @@
       <c r="AA86" s="3"/>
       <c r="AB86" s="3"/>
       <c r="AC86" s="3"/>
-    </row>
-    <row r="87" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD86" s="3"/>
+      <c r="AE86" s="3"/>
+      <c r="AF86" s="3"/>
+      <c r="AG86" s="3"/>
+      <c r="AH86" s="3"/>
+      <c r="AI86" s="3"/>
+    </row>
+    <row r="87" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A87" s="2"/>
       <c r="B87" s="2"/>
       <c r="C87" s="2"/>
@@ -3378,8 +3927,14 @@
       <c r="AA87" s="2"/>
       <c r="AB87" s="2"/>
       <c r="AC87" s="2"/>
-    </row>
-    <row r="88" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD87" s="2"/>
+      <c r="AE87" s="2"/>
+      <c r="AF87" s="2"/>
+      <c r="AG87" s="2"/>
+      <c r="AH87" s="2"/>
+      <c r="AI87" s="2"/>
+    </row>
+    <row r="88" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A88" s="3"/>
       <c r="B88" s="3"/>
       <c r="C88" s="3"/>
@@ -3409,8 +3964,14 @@
       <c r="AA88" s="3"/>
       <c r="AB88" s="3"/>
       <c r="AC88" s="3"/>
-    </row>
-    <row r="89" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD88" s="3"/>
+      <c r="AE88" s="3"/>
+      <c r="AF88" s="3"/>
+      <c r="AG88" s="3"/>
+      <c r="AH88" s="3"/>
+      <c r="AI88" s="3"/>
+    </row>
+    <row r="89" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A89" s="2"/>
       <c r="B89" s="2"/>
       <c r="C89" s="2"/>
@@ -3440,8 +4001,14 @@
       <c r="AA89" s="2"/>
       <c r="AB89" s="2"/>
       <c r="AC89" s="2"/>
-    </row>
-    <row r="90" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD89" s="2"/>
+      <c r="AE89" s="2"/>
+      <c r="AF89" s="2"/>
+      <c r="AG89" s="2"/>
+      <c r="AH89" s="2"/>
+      <c r="AI89" s="2"/>
+    </row>
+    <row r="90" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A90" s="3"/>
       <c r="B90" s="3"/>
       <c r="C90" s="3"/>
@@ -3471,8 +4038,14 @@
       <c r="AA90" s="3"/>
       <c r="AB90" s="3"/>
       <c r="AC90" s="3"/>
-    </row>
-    <row r="91" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD90" s="3"/>
+      <c r="AE90" s="3"/>
+      <c r="AF90" s="3"/>
+      <c r="AG90" s="3"/>
+      <c r="AH90" s="3"/>
+      <c r="AI90" s="3"/>
+    </row>
+    <row r="91" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A91" s="2"/>
       <c r="B91" s="2"/>
       <c r="C91" s="2"/>
@@ -3502,8 +4075,14 @@
       <c r="AA91" s="2"/>
       <c r="AB91" s="2"/>
       <c r="AC91" s="2"/>
-    </row>
-    <row r="92" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD91" s="2"/>
+      <c r="AE91" s="2"/>
+      <c r="AF91" s="2"/>
+      <c r="AG91" s="2"/>
+      <c r="AH91" s="2"/>
+      <c r="AI91" s="2"/>
+    </row>
+    <row r="92" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A92" s="3"/>
       <c r="B92" s="3"/>
       <c r="C92" s="3"/>
@@ -3533,8 +4112,14 @@
       <c r="AA92" s="3"/>
       <c r="AB92" s="3"/>
       <c r="AC92" s="3"/>
-    </row>
-    <row r="93" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD92" s="3"/>
+      <c r="AE92" s="3"/>
+      <c r="AF92" s="3"/>
+      <c r="AG92" s="3"/>
+      <c r="AH92" s="3"/>
+      <c r="AI92" s="3"/>
+    </row>
+    <row r="93" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A93" s="2"/>
       <c r="B93" s="2"/>
       <c r="C93" s="2"/>
@@ -3564,8 +4149,14 @@
       <c r="AA93" s="2"/>
       <c r="AB93" s="2"/>
       <c r="AC93" s="2"/>
-    </row>
-    <row r="94" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD93" s="2"/>
+      <c r="AE93" s="2"/>
+      <c r="AF93" s="2"/>
+      <c r="AG93" s="2"/>
+      <c r="AH93" s="2"/>
+      <c r="AI93" s="2"/>
+    </row>
+    <row r="94" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A94" s="3"/>
       <c r="B94" s="3"/>
       <c r="C94" s="3"/>
@@ -3595,8 +4186,14 @@
       <c r="AA94" s="3"/>
       <c r="AB94" s="3"/>
       <c r="AC94" s="3"/>
-    </row>
-    <row r="95" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD94" s="3"/>
+      <c r="AE94" s="3"/>
+      <c r="AF94" s="3"/>
+      <c r="AG94" s="3"/>
+      <c r="AH94" s="3"/>
+      <c r="AI94" s="3"/>
+    </row>
+    <row r="95" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A95" s="2"/>
       <c r="B95" s="2"/>
       <c r="C95" s="2"/>
@@ -3626,8 +4223,14 @@
       <c r="AA95" s="2"/>
       <c r="AB95" s="2"/>
       <c r="AC95" s="2"/>
-    </row>
-    <row r="96" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD95" s="2"/>
+      <c r="AE95" s="2"/>
+      <c r="AF95" s="2"/>
+      <c r="AG95" s="2"/>
+      <c r="AH95" s="2"/>
+      <c r="AI95" s="2"/>
+    </row>
+    <row r="96" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A96" s="3"/>
       <c r="B96" s="3"/>
       <c r="C96" s="3"/>
@@ -3657,8 +4260,14 @@
       <c r="AA96" s="3"/>
       <c r="AB96" s="3"/>
       <c r="AC96" s="3"/>
-    </row>
-    <row r="97" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD96" s="3"/>
+      <c r="AE96" s="3"/>
+      <c r="AF96" s="3"/>
+      <c r="AG96" s="3"/>
+      <c r="AH96" s="3"/>
+      <c r="AI96" s="3"/>
+    </row>
+    <row r="97" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A97" s="2"/>
       <c r="B97" s="2"/>
       <c r="C97" s="2"/>
@@ -3688,8 +4297,14 @@
       <c r="AA97" s="2"/>
       <c r="AB97" s="2"/>
       <c r="AC97" s="2"/>
-    </row>
-    <row r="98" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD97" s="2"/>
+      <c r="AE97" s="2"/>
+      <c r="AF97" s="2"/>
+      <c r="AG97" s="2"/>
+      <c r="AH97" s="2"/>
+      <c r="AI97" s="2"/>
+    </row>
+    <row r="98" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A98" s="3"/>
       <c r="B98" s="3"/>
       <c r="C98" s="3"/>
@@ -3719,8 +4334,14 @@
       <c r="AA98" s="3"/>
       <c r="AB98" s="3"/>
       <c r="AC98" s="3"/>
-    </row>
-    <row r="99" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD98" s="3"/>
+      <c r="AE98" s="3"/>
+      <c r="AF98" s="3"/>
+      <c r="AG98" s="3"/>
+      <c r="AH98" s="3"/>
+      <c r="AI98" s="3"/>
+    </row>
+    <row r="99" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A99" s="2"/>
       <c r="B99" s="2"/>
       <c r="C99" s="2"/>
@@ -3750,8 +4371,14 @@
       <c r="AA99" s="2"/>
       <c r="AB99" s="2"/>
       <c r="AC99" s="2"/>
-    </row>
-    <row r="100" spans="1:29" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="AD99" s="2"/>
+      <c r="AE99" s="2"/>
+      <c r="AF99" s="2"/>
+      <c r="AG99" s="2"/>
+      <c r="AH99" s="2"/>
+      <c r="AI99" s="2"/>
+    </row>
+    <row r="100" spans="1:35" ht="39.950000000000003" customHeight="1">
       <c r="A100" s="3"/>
       <c r="B100" s="3"/>
       <c r="C100" s="3"/>
@@ -3781,10 +4408,16 @@
       <c r="AA100" s="3"/>
       <c r="AB100" s="3"/>
       <c r="AC100" s="3"/>
+      <c r="AD100" s="3"/>
+      <c r="AE100" s="3"/>
+      <c r="AF100" s="3"/>
+      <c r="AG100" s="3"/>
+      <c r="AH100" s="3"/>
+      <c r="AI100" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:AC1"/>
+    <mergeCell ref="A1:AI1"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>